<commit_message>
Modern-OIB dataset: apply the stated selection criteria
Remove Easter sample EI9209 (MgO 7.14 wt%), the only sample in
modern_OIB.xlsx that fails the criteria now stated in the paper: SiO2,
MgO and FeOT reported with at least 6 REE; MgO > 7.5 wt%; LOI <= 5 wt%
where reported and not labelled altered; and not both Nb/U < 30 and
La/Nb >= 1.5. The dataset now has 1,800 samples from 112 locations.

Regenerate the stored full results with the paper's settings (1,651
samples inverted; thickness - seismic mean |delta| 14.01 km, was 14.02),
describe the selection in tutorials/data/README.md, update the quoted
sample counts and re-run Tutorial 3.
</commit_message>
<xml_diff>
--- a/tutorials/data/modern_OIB_precomputed/modern_OIB_sample_inversion_summary_log10.xlsx
+++ b/tutorials/data/modern_OIB_precomputed/modern_OIB_sample_inversion_summary_log10.xlsx
@@ -612,7 +612,7 @@
         <v>0.05679161669521784</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.006674096151133613</v>
+        <v>0.006674096151133612</v>
       </c>
       <c r="R2" t="n">
         <v>0.1666872937419192</v>
@@ -734,28 +734,28 @@
         <v>96.50634540601466</v>
       </c>
       <c r="C4" t="n">
-        <v>72.47120083548621</v>
+        <v>72.47120083548623</v>
       </c>
       <c r="D4" t="n">
-        <v>69.22328023585065</v>
+        <v>69.22328023585067</v>
       </c>
       <c r="E4" t="n">
-        <v>75.71912143512178</v>
+        <v>75.71912143512179</v>
       </c>
       <c r="F4" t="n">
         <v>52.28056039599736</v>
       </c>
       <c r="G4" t="n">
-        <v>58.89022515289268</v>
+        <v>58.89022515289269</v>
       </c>
       <c r="H4" t="n">
-        <v>55.12121284282219</v>
+        <v>55.1212128428222</v>
       </c>
       <c r="I4" t="n">
-        <v>62.65923746296316</v>
+        <v>62.65923746296318</v>
       </c>
       <c r="J4" t="n">
-        <v>112.8758895881982</v>
+        <v>112.8758895881983</v>
       </c>
       <c r="K4" t="n">
         <v>101.5000354776232</v>
@@ -828,13 +828,13 @@
         <v>53.71034567763792</v>
       </c>
       <c r="G5" t="n">
-        <v>57.88093625470582</v>
+        <v>57.88093625470581</v>
       </c>
       <c r="H5" t="n">
-        <v>53.31111124692188</v>
+        <v>53.31111124692187</v>
       </c>
       <c r="I5" t="n">
-        <v>62.45076126248976</v>
+        <v>62.45076126248975</v>
       </c>
       <c r="J5" t="n">
         <v>113.5895794528621</v>
@@ -882,7 +882,7 @@
         <v>1</v>
       </c>
       <c r="Y5" t="n">
-        <v>83.44793332338917</v>
+        <v>83.44793332338914</v>
       </c>
       <c r="Z5" t="n">
         <v>14</v>
@@ -907,7 +907,7 @@
         <v>114.7779297146267</v>
       </c>
       <c r="F6" t="n">
-        <v>57.99999999999999</v>
+        <v>58</v>
       </c>
       <c r="G6" t="n">
         <v>62.18606932847765</v>
@@ -943,7 +943,7 @@
         <v>0.006888620027302832</v>
       </c>
       <c r="R6" t="n">
-        <v>0.08893086517983742</v>
+        <v>0.08893086517983741</v>
       </c>
       <c r="S6" t="n">
         <v>2.3</v>
@@ -983,7 +983,7 @@
         <v>119.579621454894</v>
       </c>
       <c r="D7" t="n">
-        <v>66.41996810015851</v>
+        <v>66.41996810015848</v>
       </c>
       <c r="E7" t="n">
         <v>172.7392748096295</v>
@@ -1016,7 +1016,7 @@
         <v>0.005061656057734498</v>
       </c>
       <c r="O7" t="n">
-        <v>0.04845671931986862</v>
+        <v>0.04845671931986863</v>
       </c>
       <c r="P7" t="n">
         <v>0.05180359194843186</v>
@@ -1031,10 +1031,10 @@
         <v>1.54545356093958</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.02235808208757772</v>
+        <v>-0.02235808208757795</v>
       </c>
       <c r="U7" t="n">
-        <v>3.113265203966737</v>
+        <v>3.113265203966738</v>
       </c>
       <c r="V7" t="n">
         <v>0.03562418684073195</v>
@@ -1046,7 +1046,7 @@
         <v>1</v>
       </c>
       <c r="Y7" t="n">
-        <v>73.76808465389455</v>
+        <v>73.76808465389456</v>
       </c>
       <c r="Z7" t="n">
         <v>13</v>
@@ -1153,13 +1153,13 @@
         <v>181.6820526552546</v>
       </c>
       <c r="F9" t="n">
-        <v>74.69007729791598</v>
+        <v>74.69007729791596</v>
       </c>
       <c r="G9" t="n">
-        <v>80.97282154573196</v>
+        <v>80.97282154573195</v>
       </c>
       <c r="H9" t="n">
-        <v>69.31840599345345</v>
+        <v>69.31840599345342</v>
       </c>
       <c r="I9" t="n">
         <v>92.62723709801047</v>
@@ -1177,28 +1177,28 @@
         <v>0.01493978042115314</v>
       </c>
       <c r="N9" t="n">
-        <v>0.004075274770457048</v>
+        <v>0.004075274770457047</v>
       </c>
       <c r="O9" t="n">
-        <v>0.02936900837264863</v>
+        <v>0.02936900837264862</v>
       </c>
       <c r="P9" t="n">
-        <v>0.04132654666442856</v>
+        <v>0.04132654666442857</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.008318591710376489</v>
+        <v>0.008318591710376487</v>
       </c>
       <c r="R9" t="n">
         <v>0.1125117412319813</v>
       </c>
       <c r="S9" t="n">
-        <v>4.251885103456048</v>
+        <v>4.251885103456047</v>
       </c>
       <c r="T9" t="n">
-        <v>2.6318581744169</v>
+        <v>2.631858174416899</v>
       </c>
       <c r="U9" t="n">
-        <v>5.871912032495196</v>
+        <v>5.871912032495195</v>
       </c>
       <c r="V9" t="n">
         <v>0.01559699336049103</v>
@@ -1210,7 +1210,7 @@
         <v>1</v>
       </c>
       <c r="Y9" t="n">
-        <v>84.8595851133864</v>
+        <v>84.85958511338639</v>
       </c>
       <c r="Z9" t="n">
         <v>5</v>
@@ -1235,13 +1235,13 @@
         <v>168.9909268832168</v>
       </c>
       <c r="F10" t="n">
-        <v>53.94300308883514</v>
+        <v>53.94300308883513</v>
       </c>
       <c r="G10" t="n">
         <v>58.38359907105998</v>
       </c>
       <c r="H10" t="n">
-        <v>49.61802523552613</v>
+        <v>49.61802523552612</v>
       </c>
       <c r="I10" t="n">
         <v>67.14917290659383</v>
@@ -1268,19 +1268,19 @@
         <v>0.05258552394091844</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.008881871476444878</v>
+        <v>0.008881871476444876</v>
       </c>
       <c r="R10" t="n">
         <v>0.1516191488622755</v>
       </c>
       <c r="S10" t="n">
-        <v>3.644523391645718</v>
+        <v>3.644523391645717</v>
       </c>
       <c r="T10" t="n">
-        <v>-1.600394936322383</v>
+        <v>-1.600394936322384</v>
       </c>
       <c r="U10" t="n">
-        <v>8.889441719613819</v>
+        <v>8.889441719613817</v>
       </c>
       <c r="V10" t="n">
         <v>0.02294625795061091</v>
@@ -1292,7 +1292,7 @@
         <v>1</v>
       </c>
       <c r="Y10" t="n">
-        <v>72.42474803124571</v>
+        <v>72.4247480312457</v>
       </c>
       <c r="Z10" t="n">
         <v>9</v>
@@ -1308,10 +1308,10 @@
         <v>124.2079481465696</v>
       </c>
       <c r="C11" t="n">
-        <v>98.658112474829</v>
+        <v>98.65811247482897</v>
       </c>
       <c r="D11" t="n">
-        <v>63.87668913969005</v>
+        <v>63.87668913969001</v>
       </c>
       <c r="E11" t="n">
         <v>133.4395358099679</v>
@@ -1320,13 +1320,13 @@
         <v>67.2049640412781</v>
       </c>
       <c r="G11" t="n">
-        <v>74.23116885100677</v>
+        <v>74.23116885100676</v>
       </c>
       <c r="H11" t="n">
-        <v>55.67973820296794</v>
+        <v>55.67973820296793</v>
       </c>
       <c r="I11" t="n">
-        <v>92.7825994990456</v>
+        <v>92.78259949904559</v>
       </c>
       <c r="J11" t="n">
         <v>125.8757610546319</v>
@@ -1341,7 +1341,7 @@
         <v>0.0138361337191478</v>
       </c>
       <c r="N11" t="n">
-        <v>0.004534555335774476</v>
+        <v>0.004534555335774475</v>
       </c>
       <c r="O11" t="n">
         <v>0.02635618896782582</v>
@@ -1353,16 +1353,16 @@
         <v>0.007631242408329125</v>
       </c>
       <c r="R11" t="n">
-        <v>0.06685559230563527</v>
+        <v>0.0668555923056353</v>
       </c>
       <c r="S11" t="n">
-        <v>5.563201479764705</v>
+        <v>5.563201479764703</v>
       </c>
       <c r="T11" t="n">
         <v>1.405617497897985</v>
       </c>
       <c r="U11" t="n">
-        <v>9.720785461631424</v>
+        <v>9.720785461631422</v>
       </c>
       <c r="V11" t="n">
         <v>0.02539551007385144</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>92.91291512583655</v>
+        <v>92.91291512583656</v>
       </c>
       <c r="C12" t="n">
         <v>78.60676769238313</v>
@@ -1417,7 +1417,7 @@
         <v>95.76115925358103</v>
       </c>
       <c r="L12" t="n">
-        <v>119.4758956905086</v>
+        <v>119.4758956905087</v>
       </c>
       <c r="M12" t="n">
         <v>0.01933853031128163</v>
@@ -1429,7 +1429,7 @@
         <v>0.03737338180635742</v>
       </c>
       <c r="P12" t="n">
-        <v>0.02152271615680804</v>
+        <v>0.02152271615680803</v>
       </c>
       <c r="Q12" t="n">
         <v>0.008443110937489074</v>
@@ -1557,10 +1557,10 @@
         <v>58.06204829642347</v>
       </c>
       <c r="D14" t="n">
-        <v>52.87695814185262</v>
+        <v>52.87695814185261</v>
       </c>
       <c r="E14" t="n">
-        <v>63.24713845099432</v>
+        <v>63.24713845099433</v>
       </c>
       <c r="F14" t="n">
         <v>48.39116040999427</v>
@@ -1575,10 +1575,10 @@
         <v>59.96404233394465</v>
       </c>
       <c r="J14" t="n">
-        <v>111.9458819710189</v>
+        <v>111.9458819710188</v>
       </c>
       <c r="K14" t="n">
-        <v>99.5303270238859</v>
+        <v>99.53032702388589</v>
       </c>
       <c r="L14" t="n">
         <v>123.3347468188887</v>
@@ -1620,7 +1620,7 @@
         <v>1</v>
       </c>
       <c r="Y14" t="n">
-        <v>50.71965346943913</v>
+        <v>50.71965346943912</v>
       </c>
       <c r="Z14" t="n">
         <v>4</v>
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>91.79566972250896</v>
+        <v>91.79566972250895</v>
       </c>
       <c r="C15" t="n">
         <v>64.61630211791976</v>
@@ -1648,16 +1648,16 @@
         <v>47.81954947276964</v>
       </c>
       <c r="G15" t="n">
-        <v>55.29387556403167</v>
+        <v>55.29387556403168</v>
       </c>
       <c r="H15" t="n">
         <v>52.81783533983623</v>
       </c>
       <c r="I15" t="n">
-        <v>57.76991578822712</v>
+        <v>57.76991578822713</v>
       </c>
       <c r="J15" t="n">
-        <v>110.1996657579857</v>
+        <v>110.1996657579856</v>
       </c>
       <c r="K15" t="n">
         <v>97.68795254669956</v>
@@ -1669,10 +1669,10 @@
         <v>0.0208425712260319</v>
       </c>
       <c r="N15" t="n">
-        <v>0.00622766823024229</v>
+        <v>0.006227668230242288</v>
       </c>
       <c r="O15" t="n">
-        <v>0.04030225558428782</v>
+        <v>0.04030225558428781</v>
       </c>
       <c r="P15" t="n">
         <v>0.02275283092462708</v>
@@ -1681,16 +1681,16 @@
         <v>0.008474611527462365</v>
       </c>
       <c r="R15" t="n">
-        <v>0.06737389380953324</v>
+        <v>0.06737389380953322</v>
       </c>
       <c r="S15" t="n">
-        <v>4.567738749588193</v>
+        <v>4.567738749588192</v>
       </c>
       <c r="T15" t="n">
-        <v>3.628303411910725</v>
+        <v>3.628303411910724</v>
       </c>
       <c r="U15" t="n">
-        <v>5.50717408726566</v>
+        <v>5.507174087265659</v>
       </c>
       <c r="V15" t="n">
         <v>0.02538177042965383</v>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="Y15" t="n">
-        <v>51.82003164310311</v>
+        <v>51.82003164310309</v>
       </c>
       <c r="Z15" t="n">
         <v>4</v>
@@ -1751,7 +1751,7 @@
         <v>0.01459192116062727</v>
       </c>
       <c r="N16" t="n">
-        <v>0.004531581002127099</v>
+        <v>0.004531581002127098</v>
       </c>
       <c r="O16" t="n">
         <v>0.02778235904780866</v>
@@ -1769,7 +1769,7 @@
         <v>7.487390942616405</v>
       </c>
       <c r="T16" t="n">
-        <v>6.190819657203406</v>
+        <v>6.190819657203405</v>
       </c>
       <c r="U16" t="n">
         <v>8.783962228029404</v>
@@ -1882,22 +1882,22 @@
         <v>90.44976252960392</v>
       </c>
       <c r="C18" t="n">
-        <v>69.39183166629765</v>
+        <v>69.39183166629766</v>
       </c>
       <c r="D18" t="n">
         <v>63.73022193232423</v>
       </c>
       <c r="E18" t="n">
-        <v>75.05344140027107</v>
+        <v>75.05344140027108</v>
       </c>
       <c r="F18" t="n">
-        <v>46.80658326379905</v>
+        <v>46.80658326379906</v>
       </c>
       <c r="G18" t="n">
         <v>52.59751425120827</v>
       </c>
       <c r="H18" t="n">
-        <v>49.63918880682918</v>
+        <v>49.6391888068292</v>
       </c>
       <c r="I18" t="n">
         <v>55.55583969558735</v>
@@ -1906,22 +1906,22 @@
         <v>107.6991742782584</v>
       </c>
       <c r="K18" t="n">
-        <v>94.84418445282678</v>
+        <v>94.84418445282679</v>
       </c>
       <c r="L18" t="n">
         <v>120.0071545259141</v>
       </c>
       <c r="M18" t="n">
-        <v>0.02171335224253236</v>
+        <v>0.02171335224253237</v>
       </c>
       <c r="N18" t="n">
-        <v>0.005773488451907306</v>
+        <v>0.005773488451907307</v>
       </c>
       <c r="O18" t="n">
         <v>0.0429946745473925</v>
       </c>
       <c r="P18" t="n">
-        <v>0.0233561838904678</v>
+        <v>0.02335618389046781</v>
       </c>
       <c r="Q18" t="n">
         <v>0.008398707087313318</v>
@@ -1930,10 +1930,10 @@
         <v>0.06911605546860627</v>
       </c>
       <c r="S18" t="n">
-        <v>3.315223959852316</v>
+        <v>3.315223959852317</v>
       </c>
       <c r="T18" t="n">
-        <v>2.112211287514147</v>
+        <v>2.112211287514148</v>
       </c>
       <c r="U18" t="n">
         <v>4.518236632190486</v>
@@ -1948,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="Y18" t="n">
-        <v>52.7825106530091</v>
+        <v>52.78251065300911</v>
       </c>
       <c r="Z18" t="n">
         <v>11</v>
@@ -1964,10 +1964,10 @@
         <v>104.6618762096081</v>
       </c>
       <c r="C19" t="n">
-        <v>75.22205082800483</v>
+        <v>75.22205082800481</v>
       </c>
       <c r="D19" t="n">
-        <v>46.920422399976</v>
+        <v>46.92042239997599</v>
       </c>
       <c r="E19" t="n">
         <v>103.5236792560336</v>
@@ -1976,19 +1976,19 @@
         <v>48.3092844373551</v>
       </c>
       <c r="G19" t="n">
-        <v>56.40523641729599</v>
+        <v>56.405236417296</v>
       </c>
       <c r="H19" t="n">
-        <v>52.84988647318919</v>
+        <v>52.8498864731892</v>
       </c>
       <c r="I19" t="n">
-        <v>59.96058636140278</v>
+        <v>59.96058636140279</v>
       </c>
       <c r="J19" t="n">
-        <v>112.3267489832746</v>
+        <v>112.3267489832745</v>
       </c>
       <c r="K19" t="n">
-        <v>99.36074429544523</v>
+        <v>99.36074429544524</v>
       </c>
       <c r="L19" t="n">
         <v>125.3320443842836</v>
@@ -2000,7 +2000,7 @@
         <v>0.006172423433866985</v>
       </c>
       <c r="O19" t="n">
-        <v>0.04729704150644885</v>
+        <v>0.04729704150644884</v>
       </c>
       <c r="P19" t="n">
         <v>0.03115752915063418</v>
@@ -2009,22 +2009,22 @@
         <v>0.008476075144941692</v>
       </c>
       <c r="R19" t="n">
-        <v>0.09162800344943503</v>
+        <v>0.09162800344943499</v>
       </c>
       <c r="S19" t="n">
-        <v>5.319434689730226</v>
+        <v>5.319434689730225</v>
       </c>
       <c r="T19" t="n">
-        <v>3.172998389028068</v>
+        <v>3.172998389028067</v>
       </c>
       <c r="U19" t="n">
-        <v>7.465870990432384</v>
+        <v>7.465870990432383</v>
       </c>
       <c r="V19" t="n">
-        <v>0.02558330193662776</v>
+        <v>0.02558330193662777</v>
       </c>
       <c r="W19" t="n">
-        <v>0.02558330193662776</v>
+        <v>0.02558330193662777</v>
       </c>
       <c r="X19" t="n">
         <v>1</v>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>101.266130086404</v>
+        <v>101.2661300864041</v>
       </c>
       <c r="C20" t="n">
         <v>64.43107703902039</v>
@@ -2058,13 +2058,13 @@
         <v>56.1911753867512</v>
       </c>
       <c r="G20" t="n">
-        <v>66.3208149747817</v>
+        <v>66.32081497478171</v>
       </c>
       <c r="H20" t="n">
-        <v>60.88922255721567</v>
+        <v>60.88922255721568</v>
       </c>
       <c r="I20" t="n">
-        <v>71.75240739234773</v>
+        <v>71.75240739234775</v>
       </c>
       <c r="J20" t="n">
         <v>119.6663194637277</v>
@@ -2112,7 +2112,7 @@
         <v>1</v>
       </c>
       <c r="Y20" t="n">
-        <v>67.66582456665245</v>
+        <v>67.66582456665246</v>
       </c>
       <c r="Z20" t="n">
         <v>31</v>
@@ -2143,10 +2143,10 @@
         <v>57.95258363536225</v>
       </c>
       <c r="H21" t="n">
-        <v>50.30722625320029</v>
+        <v>50.30722625320028</v>
       </c>
       <c r="I21" t="n">
-        <v>65.59794101752422</v>
+        <v>65.59794101752421</v>
       </c>
       <c r="J21" t="n">
         <v>114.118476086044</v>
@@ -2158,22 +2158,22 @@
         <v>127.3864636955704</v>
       </c>
       <c r="M21" t="n">
-        <v>0.02403825850643148</v>
+        <v>0.02403825850643147</v>
       </c>
       <c r="N21" t="n">
         <v>0.005546281771976008</v>
       </c>
       <c r="O21" t="n">
-        <v>0.04913494192770804</v>
+        <v>0.04913494192770803</v>
       </c>
       <c r="P21" t="n">
-        <v>0.03109128323735896</v>
+        <v>0.03109128323735895</v>
       </c>
       <c r="Q21" t="n">
         <v>0.00778810863096252</v>
       </c>
       <c r="R21" t="n">
-        <v>0.08903711139513591</v>
+        <v>0.0890371113951359</v>
       </c>
       <c r="S21" t="n">
         <v>7.692972240848603</v>
@@ -2194,7 +2194,7 @@
         <v>1</v>
       </c>
       <c r="Y21" t="n">
-        <v>59.01092210360491</v>
+        <v>59.01092210360492</v>
       </c>
       <c r="Z21" t="n">
         <v>11</v>
@@ -2210,10 +2210,10 @@
         <v>135.8602942972068</v>
       </c>
       <c r="C22" t="n">
-        <v>92.78403901694946</v>
+        <v>92.78403901694945</v>
       </c>
       <c r="D22" t="n">
-        <v>56.29403101719505</v>
+        <v>56.29403101719504</v>
       </c>
       <c r="E22" t="n">
         <v>129.2740470167039</v>
@@ -2225,7 +2225,7 @@
         <v>87.05298500392666</v>
       </c>
       <c r="H22" t="n">
-        <v>70.08790478417322</v>
+        <v>70.0879047841732</v>
       </c>
       <c r="I22" t="n">
         <v>104.0180652236801</v>
@@ -2234,7 +2234,7 @@
         <v>136.9080838851283</v>
       </c>
       <c r="K22" t="n">
-        <v>127.0161529644614</v>
+        <v>127.0161529644613</v>
       </c>
       <c r="L22" t="n">
         <v>146.2172394907206</v>
@@ -2243,7 +2243,7 @@
         <v>0.01110205074839582</v>
       </c>
       <c r="N22" t="n">
-        <v>0.003728876650591809</v>
+        <v>0.003728876650591808</v>
       </c>
       <c r="O22" t="n">
         <v>0.02078391686617828</v>
@@ -2255,13 +2255,13 @@
         <v>0.007048174881677887</v>
       </c>
       <c r="R22" t="n">
-        <v>0.0628617164196045</v>
+        <v>0.06286171641960449</v>
       </c>
       <c r="S22" t="n">
         <v>11.3667265428446</v>
       </c>
       <c r="T22" t="n">
-        <v>8.61576122953857</v>
+        <v>8.615761229538567</v>
       </c>
       <c r="U22" t="n">
         <v>14.11769185615063</v>
@@ -2304,13 +2304,13 @@
         <v>69.70177221199512</v>
       </c>
       <c r="G23" t="n">
-        <v>76.19072193993105</v>
+        <v>76.19072193993104</v>
       </c>
       <c r="H23" t="n">
-        <v>54.80989488858414</v>
+        <v>54.80989488858413</v>
       </c>
       <c r="I23" t="n">
-        <v>97.57154899127796</v>
+        <v>97.57154899127795</v>
       </c>
       <c r="J23" t="n">
         <v>130.3253214709993</v>
@@ -2325,13 +2325,13 @@
         <v>0.01929272219187624</v>
       </c>
       <c r="N23" t="n">
-        <v>0.004191381108921582</v>
+        <v>0.004191381108921581</v>
       </c>
       <c r="O23" t="n">
-        <v>0.03999123812677232</v>
+        <v>0.03999123812677231</v>
       </c>
       <c r="P23" t="n">
-        <v>0.04362661307435977</v>
+        <v>0.04362661307435975</v>
       </c>
       <c r="Q23" t="n">
         <v>0.008250666767709603</v>
@@ -2358,7 +2358,7 @@
         <v>1</v>
       </c>
       <c r="Y23" t="n">
-        <v>84.70162392359829</v>
+        <v>84.70162392359826</v>
       </c>
       <c r="Z23" t="n">
         <v>6</v>
@@ -2377,7 +2377,7 @@
         <v>124.4627115780307</v>
       </c>
       <c r="D24" t="n">
-        <v>104.866405738866</v>
+        <v>104.8664057388661</v>
       </c>
       <c r="E24" t="n">
         <v>144.0590174171954</v>
@@ -2389,7 +2389,7 @@
         <v>94.31703115140942</v>
       </c>
       <c r="H24" t="n">
-        <v>70.01091169439539</v>
+        <v>70.01091169439538</v>
       </c>
       <c r="I24" t="n">
         <v>118.6231506084235</v>
@@ -2459,16 +2459,16 @@
         <v>121.8173405478261</v>
       </c>
       <c r="D25" t="n">
-        <v>74.20021503133421</v>
+        <v>74.20021503133422</v>
       </c>
       <c r="E25" t="n">
         <v>169.4344660643181</v>
       </c>
       <c r="F25" t="n">
-        <v>73.52319022210024</v>
+        <v>73.52319022210025</v>
       </c>
       <c r="G25" t="n">
-        <v>84.14379612031132</v>
+        <v>84.14379612031134</v>
       </c>
       <c r="H25" t="n">
         <v>64.16464807959524</v>
@@ -2492,7 +2492,7 @@
         <v>0.004731039964908959</v>
       </c>
       <c r="O25" t="n">
-        <v>0.03547860065581259</v>
+        <v>0.0354786006558126</v>
       </c>
       <c r="P25" t="n">
         <v>0.04456076877370196</v>
@@ -2547,16 +2547,16 @@
         <v>107.0312012667496</v>
       </c>
       <c r="F26" t="n">
-        <v>67.25184520758171</v>
+        <v>67.2518452075817</v>
       </c>
       <c r="G26" t="n">
-        <v>77.90572834852514</v>
+        <v>77.90572834852513</v>
       </c>
       <c r="H26" t="n">
-        <v>60.38945387566933</v>
+        <v>60.38945387566932</v>
       </c>
       <c r="I26" t="n">
-        <v>95.42200282138096</v>
+        <v>95.42200282138094</v>
       </c>
       <c r="J26" t="n">
         <v>129.2634457392241</v>
@@ -2577,7 +2577,7 @@
         <v>0.02176169147529149</v>
       </c>
       <c r="P26" t="n">
-        <v>0.02001117754379976</v>
+        <v>0.02001117754379975</v>
       </c>
       <c r="Q26" t="n">
         <v>0.007962955430874816</v>
@@ -2623,7 +2623,7 @@
         <v>102.8312879613113</v>
       </c>
       <c r="D27" t="n">
-        <v>66.97851889291789</v>
+        <v>66.97851889291788</v>
       </c>
       <c r="E27" t="n">
         <v>138.6840570297048</v>
@@ -2638,7 +2638,7 @@
         <v>52.66530826039178</v>
       </c>
       <c r="I27" t="n">
-        <v>71.46828813385638</v>
+        <v>71.46828813385639</v>
       </c>
       <c r="J27" t="n">
         <v>118.1181587759286</v>
@@ -2647,7 +2647,7 @@
         <v>105.4359528060389</v>
       </c>
       <c r="L27" t="n">
-        <v>131.1564501059007</v>
+        <v>131.1564501059006</v>
       </c>
       <c r="M27" t="n">
         <v>0.02341993619616747</v>
@@ -2662,19 +2662,19 @@
         <v>0.03887420296365234</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.007716864659721893</v>
+        <v>0.007716864659721894</v>
       </c>
       <c r="R27" t="n">
         <v>0.1118589307226031</v>
       </c>
       <c r="S27" t="n">
-        <v>4.800372993032844</v>
+        <v>4.800372993032845</v>
       </c>
       <c r="T27" t="n">
-        <v>1.055654679541867</v>
+        <v>1.055654679541868</v>
       </c>
       <c r="U27" t="n">
-        <v>8.545091306523821</v>
+        <v>8.545091306523823</v>
       </c>
       <c r="V27" t="n">
         <v>0.02229529141762354</v>
@@ -2686,7 +2686,7 @@
         <v>1</v>
       </c>
       <c r="Y27" t="n">
-        <v>92.81348439598358</v>
+        <v>92.81348439598359</v>
       </c>
       <c r="Z27" t="n">
         <v>22</v>
@@ -2705,22 +2705,22 @@
         <v>113.9187694983088</v>
       </c>
       <c r="D28" t="n">
-        <v>53.8805364347973</v>
+        <v>53.88053643479729</v>
       </c>
       <c r="E28" t="n">
         <v>173.9570025618204</v>
       </c>
       <c r="F28" t="n">
-        <v>72.51701362930092</v>
+        <v>72.51701362930091</v>
       </c>
       <c r="G28" t="n">
         <v>82.37790646878015</v>
       </c>
       <c r="H28" t="n">
-        <v>63.65729690628655</v>
+        <v>63.65729690628656</v>
       </c>
       <c r="I28" t="n">
-        <v>101.0985160312738</v>
+        <v>101.0985160312737</v>
       </c>
       <c r="J28" t="n">
         <v>135.8542305933526</v>
@@ -2732,16 +2732,16 @@
         <v>147.043668013467</v>
       </c>
       <c r="M28" t="n">
-        <v>0.01537041788094994</v>
+        <v>0.01537041788094993</v>
       </c>
       <c r="N28" t="n">
         <v>0.004237330054098295</v>
       </c>
       <c r="O28" t="n">
-        <v>0.03044405101811849</v>
+        <v>0.03044405101811848</v>
       </c>
       <c r="P28" t="n">
-        <v>0.04110898739532424</v>
+        <v>0.04110898739532423</v>
       </c>
       <c r="Q28" t="n">
         <v>0.009841827885032548</v>
@@ -2753,7 +2753,7 @@
         <v>9.245784638485018</v>
       </c>
       <c r="T28" t="n">
-        <v>5.081911415500614</v>
+        <v>5.081911415500613</v>
       </c>
       <c r="U28" t="n">
         <v>13.40965786146942</v>
@@ -2787,7 +2787,7 @@
         <v>108.7563474732441</v>
       </c>
       <c r="D29" t="n">
-        <v>93.72835831907635</v>
+        <v>93.72835831907636</v>
       </c>
       <c r="E29" t="n">
         <v>123.7843366274118</v>
@@ -2796,13 +2796,13 @@
         <v>62.43174433013318</v>
       </c>
       <c r="G29" t="n">
-        <v>72.05141815199376</v>
+        <v>72.05141815199374</v>
       </c>
       <c r="H29" t="n">
-        <v>59.42303069525383</v>
+        <v>59.42303069525381</v>
       </c>
       <c r="I29" t="n">
-        <v>84.67980560873369</v>
+        <v>84.67980560873367</v>
       </c>
       <c r="J29" t="n">
         <v>127.3572591570491</v>
@@ -2811,7 +2811,7 @@
         <v>114.6642062650774</v>
       </c>
       <c r="L29" t="n">
-        <v>140.496356840302</v>
+        <v>140.4963568403021</v>
       </c>
       <c r="M29" t="n">
         <v>0.02070875060511483</v>
@@ -2823,7 +2823,7 @@
         <v>0.04483176374658605</v>
       </c>
       <c r="P29" t="n">
-        <v>0.0418770763123783</v>
+        <v>0.04187707631237829</v>
       </c>
       <c r="Q29" t="n">
         <v>0.006949553412905676</v>
@@ -2832,13 +2832,13 @@
         <v>0.1143035372796286</v>
       </c>
       <c r="S29" t="n">
-        <v>7.69039990252226</v>
+        <v>7.690399902522258</v>
       </c>
       <c r="T29" t="n">
-        <v>4.791960598202603</v>
+        <v>4.791960598202601</v>
       </c>
       <c r="U29" t="n">
-        <v>10.58883920684192</v>
+        <v>10.58883920684191</v>
       </c>
       <c r="V29" t="n">
         <v>0.01893388393482081</v>
@@ -2850,7 +2850,7 @@
         <v>1</v>
       </c>
       <c r="Y29" t="n">
-        <v>83.4960861206053</v>
+        <v>83.49608612060528</v>
       </c>
       <c r="Z29" t="n">
         <v>3</v>
@@ -2890,7 +2890,7 @@
         <v>138.8238784492461</v>
       </c>
       <c r="K30" t="n">
-        <v>123.7363765864368</v>
+        <v>123.7363765864369</v>
       </c>
       <c r="L30" t="n">
         <v>153.7363765864368</v>
@@ -2932,7 +2932,7 @@
         <v>1</v>
       </c>
       <c r="Y30" t="n">
-        <v>84.8677119166632</v>
+        <v>84.86771191666321</v>
       </c>
       <c r="Z30" t="n">
         <v>1</v>
@@ -2987,7 +2987,7 @@
         <v>0.01749108322170576</v>
       </c>
       <c r="P31" t="n">
-        <v>0.01465921586999286</v>
+        <v>0.01465921586999285</v>
       </c>
       <c r="Q31" t="n">
         <v>0.008476049247776129</v>
@@ -3112,16 +3112,16 @@
         <v>135.3092344081866</v>
       </c>
       <c r="C33" t="n">
-        <v>100.278877518515</v>
+        <v>100.2788775185149</v>
       </c>
       <c r="D33" t="n">
-        <v>55.88787286508637</v>
+        <v>55.88787286508636</v>
       </c>
       <c r="E33" t="n">
-        <v>144.6698821719436</v>
+        <v>144.6698821719435</v>
       </c>
       <c r="F33" t="n">
-        <v>75.39324510837848</v>
+        <v>75.39324510837847</v>
       </c>
       <c r="G33" t="n">
         <v>85.02659325303817</v>
@@ -3142,10 +3142,10 @@
         <v>143.9120783290798</v>
       </c>
       <c r="M33" t="n">
-        <v>0.009930519663976668</v>
+        <v>0.009930519663976664</v>
       </c>
       <c r="N33" t="n">
-        <v>0.003917369592346554</v>
+        <v>0.003917369592346553</v>
       </c>
       <c r="O33" t="n">
         <v>0.01790064701184972</v>
@@ -3178,7 +3178,7 @@
         <v>1</v>
       </c>
       <c r="Y33" t="n">
-        <v>85.3690655627386</v>
+        <v>85.36906556273858</v>
       </c>
       <c r="Z33" t="n">
         <v>4</v>
@@ -3191,16 +3191,16 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>99.12103411653744</v>
+        <v>99.12103411653747</v>
       </c>
       <c r="C34" t="n">
-        <v>62.62094471548371</v>
+        <v>62.62094471548372</v>
       </c>
       <c r="D34" t="n">
         <v>57.72527555718317</v>
       </c>
       <c r="E34" t="n">
-        <v>67.51661387378425</v>
+        <v>67.51661387378427</v>
       </c>
       <c r="F34" t="n">
         <v>56.75950840251988</v>
@@ -3218,16 +3218,16 @@
         <v>119.7419888980738</v>
       </c>
       <c r="K34" t="n">
-        <v>109.5072933359214</v>
+        <v>109.5072933359215</v>
       </c>
       <c r="L34" t="n">
-        <v>129.1181498520365</v>
+        <v>129.1181498520366</v>
       </c>
       <c r="M34" t="n">
         <v>0.01355073783892626</v>
       </c>
       <c r="N34" t="n">
-        <v>0.005804932735083828</v>
+        <v>0.005804932735083829</v>
       </c>
       <c r="O34" t="n">
         <v>0.02365994718871244</v>
@@ -3236,13 +3236,13 @@
         <v>0.01690105678641155</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.008487700713363387</v>
+        <v>0.008487700713363388</v>
       </c>
       <c r="R34" t="n">
-        <v>0.05056067213872487</v>
+        <v>0.05056067213872488</v>
       </c>
       <c r="S34" t="n">
-        <v>7.626843865007106</v>
+        <v>7.626843865007108</v>
       </c>
       <c r="T34" t="n">
         <v>4.540589885300363</v>
@@ -3282,19 +3282,19 @@
         <v>77.20573682298885</v>
       </c>
       <c r="E35" t="n">
-        <v>135.6104009451749</v>
+        <v>135.610400945175</v>
       </c>
       <c r="F35" t="n">
-        <v>54.00000000000001</v>
+        <v>54</v>
       </c>
       <c r="G35" t="n">
-        <v>58.63773000829271</v>
+        <v>58.63773000829269</v>
       </c>
       <c r="H35" t="n">
-        <v>54.39972002873791</v>
+        <v>54.39972002873789</v>
       </c>
       <c r="I35" t="n">
-        <v>62.8757399878475</v>
+        <v>62.87573998784748</v>
       </c>
       <c r="J35" t="n">
         <v>114.8777879823806</v>
@@ -3306,31 +3306,31 @@
         <v>125.9224644484595</v>
       </c>
       <c r="M35" t="n">
-        <v>0.02133814225516662</v>
+        <v>0.02133814225516661</v>
       </c>
       <c r="N35" t="n">
-        <v>0.008387549406763513</v>
+        <v>0.008387549406763511</v>
       </c>
       <c r="O35" t="n">
-        <v>0.03835255685566239</v>
+        <v>0.03835255685566238</v>
       </c>
       <c r="P35" t="n">
-        <v>0.034294466525935</v>
+        <v>0.03429446652593499</v>
       </c>
       <c r="Q35" t="n">
         <v>0.007029357643170882</v>
       </c>
       <c r="R35" t="n">
-        <v>0.09548002053768678</v>
+        <v>0.09548002053768676</v>
       </c>
       <c r="S35" t="n">
-        <v>3.279794888355657</v>
+        <v>3.279794888355658</v>
       </c>
       <c r="T35" t="n">
-        <v>-0.778813192021663</v>
+        <v>-0.7788131920216639</v>
       </c>
       <c r="U35" t="n">
-        <v>7.338402968732978</v>
+        <v>7.33840296873298</v>
       </c>
       <c r="V35" t="n">
         <v>0.02185476817912438</v>
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>193.5488775268237</v>
+        <v>193.5488775268236</v>
       </c>
       <c r="C36" t="n">
         <v>184.5730426879573</v>
@@ -3364,7 +3364,7 @@
         <v>157.4742887497448</v>
       </c>
       <c r="E36" t="n">
-        <v>211.6717966261699</v>
+        <v>211.6717966261698</v>
       </c>
       <c r="F36" t="n">
         <v>57.59537247827235</v>
@@ -3394,7 +3394,7 @@
         <v>0.007700482075265423</v>
       </c>
       <c r="O36" t="n">
-        <v>0.09205788473798415</v>
+        <v>0.09205788473798417</v>
       </c>
       <c r="P36" t="n">
         <v>0.1340395223656122</v>
@@ -3409,7 +3409,7 @@
         <v>1.310969025770299</v>
       </c>
       <c r="T36" t="n">
-        <v>0.7899660060166451</v>
+        <v>0.7899660060166452</v>
       </c>
       <c r="U36" t="n">
         <v>1.831972045523953</v>
@@ -3443,7 +3443,7 @@
         <v>113.4926892474464</v>
       </c>
       <c r="D37" t="n">
-        <v>75.80948007600227</v>
+        <v>75.80948007600223</v>
       </c>
       <c r="E37" t="n">
         <v>151.1758984188905</v>
@@ -3476,10 +3476,10 @@
         <v>0.001539672045113788</v>
       </c>
       <c r="O37" t="n">
-        <v>0.03795368253252463</v>
+        <v>0.03795368253252464</v>
       </c>
       <c r="P37" t="n">
-        <v>0.04127186265175764</v>
+        <v>0.04127186265175765</v>
       </c>
       <c r="Q37" t="n">
         <v>0.006602291809028041</v>
@@ -3528,7 +3528,7 @@
         <v>115.2104805626997</v>
       </c>
       <c r="E38" t="n">
-        <v>149.7384125580661</v>
+        <v>149.738412558066</v>
       </c>
       <c r="F38" t="n">
         <v>66.76544722022706</v>
@@ -3546,7 +3546,7 @@
         <v>130.8911923486931</v>
       </c>
       <c r="K38" t="n">
-        <v>117.9407791394909</v>
+        <v>117.9407791394908</v>
       </c>
       <c r="L38" t="n">
         <v>144.1735136107177</v>
@@ -3555,7 +3555,7 @@
         <v>0.02331404421625112</v>
       </c>
       <c r="N38" t="n">
-        <v>0.004027183352827103</v>
+        <v>0.004027183352827102</v>
       </c>
       <c r="O38" t="n">
         <v>0.04963307536199259</v>
@@ -3573,7 +3573,7 @@
         <v>5.760298706978999</v>
       </c>
       <c r="T38" t="n">
-        <v>4.647399327923464</v>
+        <v>4.647399327923463</v>
       </c>
       <c r="U38" t="n">
         <v>6.873198086034535</v>
@@ -3588,7 +3588,7 @@
         <v>1</v>
       </c>
       <c r="Y38" t="n">
-        <v>97.19746392201488</v>
+        <v>97.19746392201486</v>
       </c>
       <c r="Z38" t="n">
         <v>3</v>
@@ -3698,7 +3698,7 @@
         <v>54.71577024469257</v>
       </c>
       <c r="G40" t="n">
-        <v>60.70327830250007</v>
+        <v>60.70327830250006</v>
       </c>
       <c r="H40" t="n">
         <v>52.98641615355761</v>
@@ -3722,16 +3722,16 @@
         <v>0.006972785557570459</v>
       </c>
       <c r="O40" t="n">
-        <v>0.02603279075797405</v>
+        <v>0.02603279075797404</v>
       </c>
       <c r="P40" t="n">
-        <v>0.0183042542823194</v>
+        <v>0.01830425428231939</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.008506073698365728</v>
+        <v>0.008506073698365726</v>
       </c>
       <c r="R40" t="n">
-        <v>0.0545037527325694</v>
+        <v>0.05450375273256938</v>
       </c>
       <c r="S40" t="n">
         <v>3.996447018936385</v>
@@ -3765,28 +3765,28 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>98.91039374538153</v>
+        <v>98.91039374538151</v>
       </c>
       <c r="C41" t="n">
-        <v>69.39225424059923</v>
+        <v>69.39225424059921</v>
       </c>
       <c r="D41" t="n">
-        <v>61.55676523211689</v>
+        <v>61.55676523211687</v>
       </c>
       <c r="E41" t="n">
-        <v>77.22774324908157</v>
+        <v>77.22774324908156</v>
       </c>
       <c r="F41" t="n">
         <v>53.41350747094975</v>
       </c>
       <c r="G41" t="n">
-        <v>61.53099583476489</v>
+        <v>61.53099583476488</v>
       </c>
       <c r="H41" t="n">
         <v>57.71317138983208</v>
       </c>
       <c r="I41" t="n">
-        <v>65.3488202796977</v>
+        <v>65.34882027969769</v>
       </c>
       <c r="J41" t="n">
         <v>115.4184447031574</v>
@@ -3798,31 +3798,31 @@
         <v>126.3134801606199</v>
       </c>
       <c r="M41" t="n">
-        <v>0.01633295129715287</v>
+        <v>0.01633295129715286</v>
       </c>
       <c r="N41" t="n">
-        <v>0.006227895426644957</v>
+        <v>0.006227895426644956</v>
       </c>
       <c r="O41" t="n">
         <v>0.02965052175137255</v>
       </c>
       <c r="P41" t="n">
-        <v>0.01987223011421997</v>
+        <v>0.01987223011421996</v>
       </c>
       <c r="Q41" t="n">
         <v>0.00852853804174135</v>
       </c>
       <c r="R41" t="n">
-        <v>0.05887910547151814</v>
+        <v>0.05887910547151812</v>
       </c>
       <c r="S41" t="n">
-        <v>5.350661227836063</v>
+        <v>5.350661227836062</v>
       </c>
       <c r="T41" t="n">
-        <v>3.714855666738738</v>
+        <v>3.714855666738736</v>
       </c>
       <c r="U41" t="n">
-        <v>6.986466788933389</v>
+        <v>6.986466788933387</v>
       </c>
       <c r="V41" t="n">
         <v>0.01471742242987522</v>
@@ -3834,7 +3834,7 @@
         <v>1</v>
       </c>
       <c r="Y41" t="n">
-        <v>76.15793456630149</v>
+        <v>76.15793456630148</v>
       </c>
       <c r="Z41" t="n">
         <v>21</v>
@@ -3862,13 +3862,13 @@
         <v>48.8395940195639</v>
       </c>
       <c r="G42" t="n">
-        <v>55.09396935508055</v>
+        <v>55.09396935508056</v>
       </c>
       <c r="H42" t="n">
         <v>51.70827498465975</v>
       </c>
       <c r="I42" t="n">
-        <v>58.47966372550136</v>
+        <v>58.47966372550137</v>
       </c>
       <c r="J42" t="n">
         <v>109.7212418994434</v>
@@ -3880,7 +3880,7 @@
         <v>121.3694068574073</v>
       </c>
       <c r="M42" t="n">
-        <v>0.01985951694492466</v>
+        <v>0.01985951694492467</v>
       </c>
       <c r="N42" t="n">
         <v>0.005551259652733669</v>
@@ -3929,79 +3929,79 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>154.5144348888715</v>
+        <v>160.7056196661262</v>
       </c>
       <c r="C43" t="n">
-        <v>148.6305648986034</v>
+        <v>153.7663035579546</v>
       </c>
       <c r="D43" t="n">
-        <v>94.92253858389762</v>
+        <v>96.94582381877021</v>
       </c>
       <c r="E43" t="n">
-        <v>202.3385912133092</v>
+        <v>210.5867832971389</v>
       </c>
       <c r="F43" t="n">
-        <v>40.72836874424947</v>
+        <v>42.29405984925105</v>
       </c>
       <c r="G43" t="n">
-        <v>42.34643299157318</v>
+        <v>44.20237177899824</v>
       </c>
       <c r="H43" t="n">
-        <v>34.923508901722</v>
+        <v>37.69570395144809</v>
       </c>
       <c r="I43" t="n">
-        <v>49.76935708142436</v>
+        <v>50.70903960654839</v>
       </c>
       <c r="J43" t="n">
-        <v>105.9932159624826</v>
+        <v>108.1228358399224</v>
       </c>
       <c r="K43" t="n">
-        <v>87.84665706709049</v>
+        <v>89.70716270873388</v>
       </c>
       <c r="L43" t="n">
-        <v>125.5274826954267</v>
+        <v>127.6894941295561</v>
       </c>
       <c r="M43" t="n">
-        <v>0.05068921935664087</v>
+        <v>0.0514606270285389</v>
       </c>
       <c r="N43" t="n">
-        <v>0.007771888168972855</v>
+        <v>0.008483606689796931</v>
       </c>
       <c r="O43" t="n">
-        <v>0.104334921425387</v>
+        <v>0.1047011673878947</v>
       </c>
       <c r="P43" t="n">
-        <v>0.1185919122878046</v>
+        <v>0.1296776232529298</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.009250524675611676</v>
+        <v>0.009712683337974025</v>
       </c>
       <c r="R43" t="n">
-        <v>0.3610965303316556</v>
+        <v>0.3959695772179068</v>
       </c>
       <c r="S43" t="n">
-        <v>0.8748340176063083</v>
+        <v>1.03176137480824</v>
       </c>
       <c r="T43" t="n">
-        <v>-0.378976559026345</v>
+        <v>-0.2690543005223529</v>
       </c>
       <c r="U43" t="n">
-        <v>2.128644594238962</v>
+        <v>2.332577050138832</v>
       </c>
       <c r="V43" t="n">
-        <v>0.02131319862989053</v>
+        <v>0.02285130053902447</v>
       </c>
       <c r="W43" t="n">
-        <v>0.02131319862989053</v>
+        <v>0.02285130053902447</v>
       </c>
       <c r="X43" t="n">
         <v>1</v>
       </c>
       <c r="Y43" t="n">
-        <v>45.79981496981414</v>
+        <v>45.97671130718118</v>
       </c>
       <c r="Z43" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44">
@@ -4011,19 +4011,19 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>244.0602851865133</v>
+        <v>244.0602851865132</v>
       </c>
       <c r="C44" t="n">
-        <v>227.0541243044931</v>
+        <v>227.054124304493</v>
       </c>
       <c r="D44" t="n">
-        <v>149.490015528564</v>
+        <v>149.4900155285639</v>
       </c>
       <c r="E44" t="n">
         <v>304.6182330804222</v>
       </c>
       <c r="F44" t="n">
-        <v>37.06982780195974</v>
+        <v>37.06982780195973</v>
       </c>
       <c r="G44" t="n">
         <v>41.7465220445153</v>
@@ -4038,16 +4038,16 @@
         <v>117.8150986626923</v>
       </c>
       <c r="K44" t="n">
-        <v>92.93190360885983</v>
+        <v>92.9319036088598</v>
       </c>
       <c r="L44" t="n">
-        <v>146.2682951298411</v>
+        <v>146.268295129841</v>
       </c>
       <c r="M44" t="n">
-        <v>0.08615193147646812</v>
+        <v>0.0861519314764681</v>
       </c>
       <c r="N44" t="n">
-        <v>0.01168876049103536</v>
+        <v>0.01168876049103535</v>
       </c>
       <c r="O44" t="n">
         <v>0.1707795314908308</v>
@@ -4056,7 +4056,7 @@
         <v>0.3931311574715851</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.009681571033590203</v>
+        <v>0.009681571033590202</v>
       </c>
       <c r="R44" t="n">
         <v>1.227468398195795</v>
@@ -4105,22 +4105,22 @@
         <v>154.6776682511037</v>
       </c>
       <c r="F45" t="n">
-        <v>29.75695700154754</v>
+        <v>29.75695700154753</v>
       </c>
       <c r="G45" t="n">
-        <v>29.75695700154754</v>
+        <v>29.75695700154753</v>
       </c>
       <c r="H45" t="n">
-        <v>27.77177940221209</v>
+        <v>27.77177940221208</v>
       </c>
       <c r="I45" t="n">
-        <v>31.74213460088298</v>
+        <v>31.74213460088297</v>
       </c>
       <c r="J45" t="n">
-        <v>96.5478054050558</v>
+        <v>96.54780540505578</v>
       </c>
       <c r="K45" t="n">
-        <v>76.68044680170748</v>
+        <v>76.68044680170745</v>
       </c>
       <c r="L45" t="n">
         <v>117.8019683009337</v>
@@ -4129,7 +4129,7 @@
         <v>0.05995634019834736</v>
       </c>
       <c r="N45" t="n">
-        <v>0.007347788636964086</v>
+        <v>0.007347788636964085</v>
       </c>
       <c r="O45" t="n">
         <v>0.1260093142937689</v>
@@ -4138,19 +4138,19 @@
         <v>0.1020203975475383</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.006520851941215646</v>
+        <v>0.006520851941215644</v>
       </c>
       <c r="R45" t="n">
-        <v>0.3070092458635797</v>
+        <v>0.3070092458635796</v>
       </c>
       <c r="S45" t="n">
-        <v>-92.19619625193442</v>
+        <v>-92.1961962519344</v>
       </c>
       <c r="T45" t="n">
-        <v>-94.67766825110373</v>
+        <v>-94.6776682511037</v>
       </c>
       <c r="U45" t="n">
-        <v>-89.71472425276512</v>
+        <v>-89.71472425276509</v>
       </c>
       <c r="V45" t="n">
         <v>0.01252580570683018</v>
@@ -4162,7 +4162,7 @@
         <v>1</v>
       </c>
       <c r="Y45" t="n">
-        <v>44.09093066736531</v>
+        <v>44.09093066736529</v>
       </c>
       <c r="Z45" t="n">
         <v>2</v>
@@ -4193,7 +4193,7 @@
         <v>30.81054819447498</v>
       </c>
       <c r="H46" t="n">
-        <v>29.66304850131349</v>
+        <v>29.6630485013135</v>
       </c>
       <c r="I46" t="n">
         <v>31.95804788763647</v>
@@ -4214,7 +4214,7 @@
         <v>0.01766162580385281</v>
       </c>
       <c r="O46" t="n">
-        <v>0.222109396729509</v>
+        <v>0.2221093967295091</v>
       </c>
       <c r="P46" t="n">
         <v>0.7113683942674621</v>
@@ -4223,7 +4223,7 @@
         <v>0.005786350452980448</v>
       </c>
       <c r="R46" t="n">
-        <v>2.275666055225475</v>
+        <v>2.275666055225476</v>
       </c>
       <c r="S46" t="n">
         <v>4.384732366997281</v>
@@ -4260,7 +4260,7 @@
         <v>104.8614981418015</v>
       </c>
       <c r="C47" t="n">
-        <v>91.66348153863935</v>
+        <v>91.66348153863933</v>
       </c>
       <c r="D47" t="n">
         <v>66.13749817840906</v>
@@ -4281,7 +4281,7 @@
         <v>34.27281622452711</v>
       </c>
       <c r="J47" t="n">
-        <v>94.2700239846741</v>
+        <v>94.27002398467411</v>
       </c>
       <c r="K47" t="n">
         <v>76.59715541860709</v>
@@ -4293,16 +4293,16 @@
         <v>0.04485098632840805</v>
       </c>
       <c r="N47" t="n">
-        <v>0.004802183960522926</v>
+        <v>0.004802183960522927</v>
       </c>
       <c r="O47" t="n">
-        <v>0.09735036240635836</v>
+        <v>0.09735036240635835</v>
       </c>
       <c r="P47" t="n">
-        <v>0.05055813293140771</v>
+        <v>0.0505581329314077</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.00665853702492561</v>
+        <v>0.006658537024925611</v>
       </c>
       <c r="R47" t="n">
         <v>0.1451098460736416</v>
@@ -4326,7 +4326,7 @@
         <v>1</v>
       </c>
       <c r="Y47" t="n">
-        <v>45.65750934973565</v>
+        <v>45.65750934973566</v>
       </c>
       <c r="Z47" t="n">
         <v>11</v>
@@ -4363,7 +4363,7 @@
         <v>45.84292052353373</v>
       </c>
       <c r="J48" t="n">
-        <v>104.265933853481</v>
+        <v>104.2659338534809</v>
       </c>
       <c r="K48" t="n">
         <v>86.49915665431766</v>
@@ -4390,13 +4390,13 @@
         <v>0.2414957114730361</v>
       </c>
       <c r="S48" t="n">
-        <v>-11.39841079409587</v>
+        <v>-11.39841079409586</v>
       </c>
       <c r="T48" t="n">
-        <v>-32.15731900505686</v>
+        <v>-32.15731900505685</v>
       </c>
       <c r="U48" t="n">
-        <v>9.360497416865117</v>
+        <v>9.360497416865121</v>
       </c>
       <c r="V48" t="n">
         <v>0.009915095034861163</v>
@@ -4424,10 +4424,10 @@
         <v>96.43974961360426</v>
       </c>
       <c r="C49" t="n">
-        <v>95.72473512930839</v>
+        <v>95.7247351293084</v>
       </c>
       <c r="D49" t="n">
-        <v>85.80239072883408</v>
+        <v>85.8023907288341</v>
       </c>
       <c r="E49" t="n">
         <v>105.6470795297827</v>
@@ -4445,10 +4445,10 @@
         <v>38.00627704238198</v>
       </c>
       <c r="J49" t="n">
-        <v>92.99873274362308</v>
+        <v>92.99873274362307</v>
       </c>
       <c r="K49" t="n">
-        <v>76.82170417299547</v>
+        <v>76.82170417299545</v>
       </c>
       <c r="L49" t="n">
         <v>109.7253450885962</v>
@@ -4460,7 +4460,7 @@
         <v>0.006118346031344804</v>
       </c>
       <c r="O49" t="n">
-        <v>0.07957288155003266</v>
+        <v>0.07957288155003263</v>
       </c>
       <c r="P49" t="n">
         <v>0.0403094148202074</v>
@@ -4490,7 +4490,7 @@
         <v>1</v>
       </c>
       <c r="Y49" t="n">
-        <v>44.51217904035592</v>
+        <v>44.51217904035593</v>
       </c>
       <c r="Z49" t="n">
         <v>8</v>
@@ -4533,7 +4533,7 @@
         <v>78.67754045169829</v>
       </c>
       <c r="L50" t="n">
-        <v>126.6676315287222</v>
+        <v>126.6676315287221</v>
       </c>
       <c r="M50" t="n">
         <v>0.08304258953477826</v>
@@ -4551,7 +4551,7 @@
         <v>0.008195851923048458</v>
       </c>
       <c r="R50" t="n">
-        <v>0.7355001850335012</v>
+        <v>0.7355001850335013</v>
       </c>
       <c r="S50" t="n">
         <v>-94.149187201214</v>
@@ -4588,7 +4588,7 @@
         <v>119.6701652593349</v>
       </c>
       <c r="C51" t="n">
-        <v>113.4917470586419</v>
+        <v>113.491747058642</v>
       </c>
       <c r="D51" t="n">
         <v>93.18802325046022</v>
@@ -4612,13 +4612,13 @@
         <v>100.1333267424856</v>
       </c>
       <c r="K51" t="n">
-        <v>84.44173621133523</v>
+        <v>84.44173621133524</v>
       </c>
       <c r="L51" t="n">
         <v>117.2453656281615</v>
       </c>
       <c r="M51" t="n">
-        <v>0.03943915054282856</v>
+        <v>0.03943915054282857</v>
       </c>
       <c r="N51" t="n">
         <v>0.006392293281950366</v>
@@ -4633,7 +4633,7 @@
         <v>0.007190843692232962</v>
       </c>
       <c r="R51" t="n">
-        <v>0.1563706145566645</v>
+        <v>0.1563706145566644</v>
       </c>
       <c r="S51" t="n">
         <v>-10.29704148176904</v>
@@ -4755,7 +4755,7 @@
         <v>136.2120897642538</v>
       </c>
       <c r="D53" t="n">
-        <v>68.5426925462137</v>
+        <v>68.54269254621369</v>
       </c>
       <c r="E53" t="n">
         <v>203.8814869822938</v>
@@ -4797,7 +4797,7 @@
         <v>0.006181882865083597</v>
       </c>
       <c r="R53" t="n">
-        <v>0.4669510933177402</v>
+        <v>0.4669510933177401</v>
       </c>
       <c r="S53" t="n">
         <v>-9.827985563563715</v>
@@ -4818,7 +4818,7 @@
         <v>1</v>
       </c>
       <c r="Y53" t="n">
-        <v>44.24732793380759</v>
+        <v>44.24732793380758</v>
       </c>
       <c r="Z53" t="n">
         <v>19</v>
@@ -4882,13 +4882,13 @@
         <v>0.5474523679392568</v>
       </c>
       <c r="S54" t="n">
-        <v>-38.73257974561326</v>
+        <v>-38.73257974561325</v>
       </c>
       <c r="T54" t="n">
         <v>-76.82863972683617</v>
       </c>
       <c r="U54" t="n">
-        <v>-0.6365197643903429</v>
+        <v>-0.6365197643903358</v>
       </c>
       <c r="V54" t="n">
         <v>0.02038125635135012</v>
@@ -4913,16 +4913,16 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>100</v>
+        <v>99.99999999999999</v>
       </c>
       <c r="C55" t="n">
-        <v>52.95921353046781</v>
+        <v>52.95921353046779</v>
       </c>
       <c r="D55" t="n">
+        <v>52.95921353046779</v>
+      </c>
+      <c r="E55" t="n">
         <v>52.9592135304678</v>
-      </c>
-      <c r="E55" t="n">
-        <v>52.95921353046781</v>
       </c>
       <c r="F55" t="n">
         <v>24</v>
@@ -4958,7 +4958,7 @@
         <v>0.04670668145766002</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.0062252735235153</v>
+        <v>0.006225273523515298</v>
       </c>
       <c r="R55" t="n">
         <v>0.1311037203693172</v>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>169.363633118192</v>
+        <v>169.3636331181919</v>
       </c>
       <c r="C56" t="n">
         <v>156.3387684642065</v>
@@ -5040,7 +5040,7 @@
         <v>0.1439904224957386</v>
       </c>
       <c r="Q56" t="n">
-        <v>0.007639193285021577</v>
+        <v>0.007639193285021578</v>
       </c>
       <c r="R56" t="n">
         <v>0.4387467326383899</v>
@@ -5064,7 +5064,7 @@
         <v>1</v>
       </c>
       <c r="Y56" t="n">
-        <v>44.14580585644439</v>
+        <v>44.1458058564444</v>
       </c>
       <c r="Z56" t="n">
         <v>46</v>
@@ -5119,13 +5119,13 @@
         <v>0.1775903071684828</v>
       </c>
       <c r="P57" t="n">
-        <v>0.3068327696315015</v>
+        <v>0.3068327696315014</v>
       </c>
       <c r="Q57" t="n">
         <v>0.01538670081711318</v>
       </c>
       <c r="R57" t="n">
-        <v>0.9993076211109189</v>
+        <v>0.9993076211109188</v>
       </c>
       <c r="S57" t="n">
         <v>-100</v>
@@ -5162,10 +5162,10 @@
         <v>123.8092296369958</v>
       </c>
       <c r="C58" t="n">
-        <v>86.53939772973868</v>
+        <v>86.5393977297387</v>
       </c>
       <c r="D58" t="n">
-        <v>60.08269361712714</v>
+        <v>60.08269361712715</v>
       </c>
       <c r="E58" t="n">
         <v>112.9961018423502</v>
@@ -5192,7 +5192,7 @@
         <v>137.4908155435125</v>
       </c>
       <c r="M58" t="n">
-        <v>0.01410270611007378</v>
+        <v>0.01410270611007377</v>
       </c>
       <c r="N58" t="n">
         <v>0.004750069424168525</v>
@@ -5213,7 +5213,7 @@
         <v>8.25153525997295</v>
       </c>
       <c r="T58" t="n">
-        <v>5.735526872311975</v>
+        <v>5.735526872311974</v>
       </c>
       <c r="U58" t="n">
         <v>10.76754364763393</v>
@@ -5253,16 +5253,16 @@
         <v>243.604741481936</v>
       </c>
       <c r="F59" t="n">
-        <v>58.96507727751418</v>
+        <v>58.96507727751419</v>
       </c>
       <c r="G59" t="n">
-        <v>58.96507727751418</v>
+        <v>58.96507727751419</v>
       </c>
       <c r="H59" t="n">
-        <v>49.97104933034797</v>
+        <v>49.97104933034798</v>
       </c>
       <c r="I59" t="n">
-        <v>67.95910522468039</v>
+        <v>67.9591052246804</v>
       </c>
       <c r="J59" t="n">
         <v>121.0124433446541</v>
@@ -5274,10 +5274,10 @@
         <v>139.5983929892861</v>
       </c>
       <c r="M59" t="n">
-        <v>0.03854596904450616</v>
+        <v>0.03854596904450617</v>
       </c>
       <c r="N59" t="n">
-        <v>0.005942548110854181</v>
+        <v>0.005942548110854182</v>
       </c>
       <c r="O59" t="n">
         <v>0.08044114619963952</v>
@@ -5310,7 +5310,7 @@
         <v>1</v>
       </c>
       <c r="Y59" t="n">
-        <v>61.40772880652974</v>
+        <v>61.40772880652975</v>
       </c>
       <c r="Z59" t="n">
         <v>6</v>
@@ -5326,16 +5326,16 @@
         <v>172.7840701361059</v>
       </c>
       <c r="C60" t="n">
-        <v>141.2879438529776</v>
+        <v>141.2879438529777</v>
       </c>
       <c r="D60" t="n">
-        <v>113.6533440719036</v>
+        <v>113.6533440719037</v>
       </c>
       <c r="E60" t="n">
         <v>168.9225436340516</v>
       </c>
       <c r="F60" t="n">
-        <v>52.40155740838307</v>
+        <v>52.40155740838308</v>
       </c>
       <c r="G60" t="n">
         <v>61.06299213624335</v>
@@ -5344,7 +5344,7 @@
         <v>51.89197015290318</v>
       </c>
       <c r="I60" t="n">
-        <v>70.23401411958352</v>
+        <v>70.23401411958353</v>
       </c>
       <c r="J60" t="n">
         <v>122.975793037996</v>
@@ -5359,10 +5359,10 @@
         <v>0.04298100557312105</v>
       </c>
       <c r="N60" t="n">
-        <v>0.005724142155820646</v>
+        <v>0.005724142155820648</v>
       </c>
       <c r="O60" t="n">
-        <v>0.09070860793948629</v>
+        <v>0.09070860793948628</v>
       </c>
       <c r="P60" t="n">
         <v>0.107029810561664</v>
@@ -5414,19 +5414,19 @@
         <v>178.1599281259955</v>
       </c>
       <c r="E61" t="n">
-        <v>227.3014034630007</v>
+        <v>227.3014034630006</v>
       </c>
       <c r="F61" t="n">
-        <v>56.93686830638941</v>
+        <v>56.9368683063894</v>
       </c>
       <c r="G61" t="n">
-        <v>56.93686830638941</v>
+        <v>56.9368683063894</v>
       </c>
       <c r="H61" t="n">
         <v>50.87717188223711</v>
       </c>
       <c r="I61" t="n">
-        <v>62.9965647305417</v>
+        <v>62.99656473054169</v>
       </c>
       <c r="J61" t="n">
         <v>121.1855539279188</v>
@@ -5441,7 +5441,7 @@
         <v>0.04870683165331807</v>
       </c>
       <c r="N61" t="n">
-        <v>0.008190674115829986</v>
+        <v>0.008190674115829985</v>
       </c>
       <c r="O61" t="n">
         <v>0.1002672482904071</v>
@@ -5453,7 +5453,7 @@
         <v>0.01456432534408538</v>
       </c>
       <c r="R61" t="n">
-        <v>0.4608359967526284</v>
+        <v>0.4608359967526283</v>
       </c>
       <c r="S61" t="n">
         <v>0</v>
@@ -5465,16 +5465,16 @@
         <v>0</v>
       </c>
       <c r="V61" t="n">
-        <v>0.05197217035017356</v>
+        <v>0.05197217035017355</v>
       </c>
       <c r="W61" t="n">
-        <v>0.05197217035017356</v>
+        <v>0.05197217035017355</v>
       </c>
       <c r="X61" t="n">
         <v>1</v>
       </c>
       <c r="Y61" t="n">
-        <v>80.11002019892018</v>
+        <v>80.11002019892017</v>
       </c>
       <c r="Z61" t="n">
         <v>5</v>
@@ -5499,7 +5499,7 @@
         <v>146.4646254925691</v>
       </c>
       <c r="F62" t="n">
-        <v>62.11991753032571</v>
+        <v>62.11991753032572</v>
       </c>
       <c r="G62" t="n">
         <v>68.23857078494049</v>
@@ -5520,10 +5520,10 @@
         <v>133.2401192545217</v>
       </c>
       <c r="M62" t="n">
-        <v>0.01747876712053072</v>
+        <v>0.01747876712053071</v>
       </c>
       <c r="N62" t="n">
-        <v>0.006197211202486231</v>
+        <v>0.006197211202486229</v>
       </c>
       <c r="O62" t="n">
         <v>0.03239107761552912</v>
@@ -5532,25 +5532,25 @@
         <v>0.0323489851366343</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.007815156749513979</v>
+        <v>0.007815156749513977</v>
       </c>
       <c r="R62" t="n">
         <v>0.09046073542502631</v>
       </c>
       <c r="S62" t="n">
-        <v>4.487040565204983</v>
+        <v>4.487040565204982</v>
       </c>
       <c r="T62" t="n">
-        <v>0.7844985008378442</v>
+        <v>0.7844985008378433</v>
       </c>
       <c r="U62" t="n">
-        <v>8.189582629572122</v>
+        <v>8.18958262957212</v>
       </c>
       <c r="V62" t="n">
-        <v>0.02982990866462304</v>
+        <v>0.02982990866462305</v>
       </c>
       <c r="W62" t="n">
-        <v>0.02982990866462304</v>
+        <v>0.02982990866462305</v>
       </c>
       <c r="X62" t="n">
         <v>1</v>
@@ -5593,7 +5593,7 @@
         <v>61.60560937351703</v>
       </c>
       <c r="J63" t="n">
-        <v>120.3653072430193</v>
+        <v>120.3653072430192</v>
       </c>
       <c r="K63" t="n">
         <v>102.2750647928757</v>
@@ -5617,13 +5617,13 @@
         <v>0.01246657725783677</v>
       </c>
       <c r="R63" t="n">
-        <v>0.4134306666076328</v>
+        <v>0.4134306666076329</v>
       </c>
       <c r="S63" t="n">
-        <v>2.348684785327081</v>
+        <v>2.34868478532708</v>
       </c>
       <c r="T63" t="n">
-        <v>0.6908642858660992</v>
+        <v>0.6908642858660987</v>
       </c>
       <c r="U63" t="n">
         <v>4.006505284788062</v>
@@ -5651,7 +5651,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>184.6340587825744</v>
+        <v>184.6340587825745</v>
       </c>
       <c r="C64" t="n">
         <v>162.8707570035273</v>
@@ -5666,13 +5666,13 @@
         <v>53.06153411839063</v>
       </c>
       <c r="G64" t="n">
-        <v>59.0464421076286</v>
+        <v>59.04644210762861</v>
       </c>
       <c r="H64" t="n">
-        <v>55.19417319792194</v>
+        <v>55.19417319792195</v>
       </c>
       <c r="I64" t="n">
-        <v>62.89871101733526</v>
+        <v>62.89871101733527</v>
       </c>
       <c r="J64" t="n">
         <v>121.9231797679321</v>
@@ -5687,10 +5687,10 @@
         <v>0.04696993285560056</v>
       </c>
       <c r="N64" t="n">
-        <v>0.007409711920525725</v>
+        <v>0.007409711920525726</v>
       </c>
       <c r="O64" t="n">
-        <v>0.09713975143660351</v>
+        <v>0.0971397514366035</v>
       </c>
       <c r="P64" t="n">
         <v>0.1199407924179182</v>
@@ -5699,7 +5699,7 @@
         <v>0.0122556408583345</v>
       </c>
       <c r="R64" t="n">
-        <v>0.3621940319672777</v>
+        <v>0.3621940319672776</v>
       </c>
       <c r="S64" t="n">
         <v>3.814816856971745</v>
@@ -5720,7 +5720,7 @@
         <v>1</v>
       </c>
       <c r="Y64" t="n">
-        <v>75.41005043715167</v>
+        <v>75.41005043715165</v>
       </c>
       <c r="Z64" t="n">
         <v>21</v>
@@ -5739,25 +5739,25 @@
         <v>183.8007852445325</v>
       </c>
       <c r="D65" t="n">
-        <v>159.2861140143192</v>
+        <v>159.2861140143191</v>
       </c>
       <c r="E65" t="n">
         <v>208.3154564747458</v>
       </c>
       <c r="F65" t="n">
-        <v>53.22633868008548</v>
+        <v>53.22633868008547</v>
       </c>
       <c r="G65" t="n">
-        <v>57.29271863009463</v>
+        <v>57.29271863009462</v>
       </c>
       <c r="H65" t="n">
-        <v>52.74239807924897</v>
+        <v>52.74239807924896</v>
       </c>
       <c r="I65" t="n">
-        <v>61.84303918094029</v>
+        <v>61.84303918094028</v>
       </c>
       <c r="J65" t="n">
-        <v>122.0475123878296</v>
+        <v>122.0475123878295</v>
       </c>
       <c r="K65" t="n">
         <v>103.6285438794018</v>
@@ -5766,7 +5766,7 @@
         <v>142.2418006919313</v>
       </c>
       <c r="M65" t="n">
-        <v>0.05171630736287239</v>
+        <v>0.05171630736287238</v>
       </c>
       <c r="N65" t="n">
         <v>0.008895403026997374</v>
@@ -5775,22 +5775,22 @@
         <v>0.1052859425178102</v>
       </c>
       <c r="P65" t="n">
-        <v>0.154875155518502</v>
+        <v>0.1548751555185019</v>
       </c>
       <c r="Q65" t="n">
         <v>0.01411291280493031</v>
       </c>
       <c r="R65" t="n">
-        <v>0.4694891616563374</v>
+        <v>0.4694891616563373</v>
       </c>
       <c r="S65" t="n">
-        <v>2.487298992885299</v>
+        <v>2.487298992885298</v>
       </c>
       <c r="T65" t="n">
-        <v>0.6429962543519014</v>
+        <v>0.6429962543519012</v>
       </c>
       <c r="U65" t="n">
-        <v>4.331601731418696</v>
+        <v>4.331601731418695</v>
       </c>
       <c r="V65" t="n">
         <v>0.01335271853275777</v>
@@ -5802,7 +5802,7 @@
         <v>1</v>
       </c>
       <c r="Y65" t="n">
-        <v>81.36371972812661</v>
+        <v>81.3637197281266</v>
       </c>
       <c r="Z65" t="n">
         <v>136</v>
@@ -5830,13 +5830,13 @@
         <v>53.79145154446059</v>
       </c>
       <c r="G66" t="n">
-        <v>56.68061878271442</v>
+        <v>56.6806187827144</v>
       </c>
       <c r="H66" t="n">
-        <v>50.09113905318471</v>
+        <v>50.09113905318469</v>
       </c>
       <c r="I66" t="n">
-        <v>63.27009851224413</v>
+        <v>63.2700985122441</v>
       </c>
       <c r="J66" t="n">
         <v>127.5630570219946</v>
@@ -5851,7 +5851,7 @@
         <v>0.06811966759963971</v>
       </c>
       <c r="N66" t="n">
-        <v>0.009072272114105823</v>
+        <v>0.009072272114105821</v>
       </c>
       <c r="O66" t="n">
         <v>0.1368787410982058</v>
@@ -5860,16 +5860,16 @@
         <v>0.3087801010707348</v>
       </c>
       <c r="Q66" t="n">
-        <v>0.01433208589084291</v>
+        <v>0.0143320858908429</v>
       </c>
       <c r="R66" t="n">
-        <v>0.9303474099860337</v>
+        <v>0.9303474099860335</v>
       </c>
       <c r="S66" t="n">
         <v>1.667790454023701</v>
       </c>
       <c r="T66" t="n">
-        <v>0.6439838278831624</v>
+        <v>0.6439838278831627</v>
       </c>
       <c r="U66" t="n">
         <v>2.691597080164239</v>
@@ -5884,7 +5884,7 @@
         <v>1</v>
       </c>
       <c r="Y66" t="n">
-        <v>82.93364180923059</v>
+        <v>82.93364180923058</v>
       </c>
       <c r="Z66" t="n">
         <v>46</v>
@@ -5903,10 +5903,10 @@
         <v>203.9804775011341</v>
       </c>
       <c r="D67" t="n">
-        <v>136.6983827816145</v>
+        <v>136.6983827816144</v>
       </c>
       <c r="E67" t="n">
-        <v>271.2625722206537</v>
+        <v>271.2625722206538</v>
       </c>
       <c r="F67" t="n">
         <v>50.8239290628899</v>
@@ -5933,7 +5933,7 @@
         <v>0.05680990488571173</v>
       </c>
       <c r="N67" t="n">
-        <v>0.009337065358427909</v>
+        <v>0.009337065358427907</v>
       </c>
       <c r="O67" t="n">
         <v>0.1150541382810456</v>
@@ -5979,7 +5979,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>187.2302147309323</v>
+        <v>187.2302147309324</v>
       </c>
       <c r="C68" t="n">
         <v>147.6044706756228</v>
@@ -5997,7 +5997,7 @@
         <v>113.3120001471554</v>
       </c>
       <c r="H68" t="n">
-        <v>101.7429718182577</v>
+        <v>101.7429718182578</v>
       </c>
       <c r="I68" t="n">
         <v>124.8810284760531</v>
@@ -6006,13 +6006,13 @@
         <v>158.6401362092208</v>
       </c>
       <c r="K68" t="n">
-        <v>149.6229334309502</v>
+        <v>149.6229334309503</v>
       </c>
       <c r="L68" t="n">
-        <v>167.3674495707543</v>
+        <v>167.3674495707544</v>
       </c>
       <c r="M68" t="n">
-        <v>0.008088847922436245</v>
+        <v>0.008088847922436247</v>
       </c>
       <c r="N68" t="n">
         <v>0.002898777441228873</v>
@@ -6021,34 +6021,34 @@
         <v>0.01504936301469817</v>
       </c>
       <c r="P68" t="n">
-        <v>0.02866510781672575</v>
+        <v>0.02866510781672576</v>
       </c>
       <c r="Q68" t="n">
-        <v>0.008724851213324177</v>
+        <v>0.008724851213324178</v>
       </c>
       <c r="R68" t="n">
         <v>0.07855574055494433</v>
       </c>
       <c r="S68" t="n">
-        <v>12.89328275829246</v>
+        <v>12.89328275829247</v>
       </c>
       <c r="T68" t="n">
-        <v>9.997530147049034</v>
+        <v>9.997530147049037</v>
       </c>
       <c r="U68" t="n">
         <v>15.7890353695359</v>
       </c>
       <c r="V68" t="n">
-        <v>0.043129562604745</v>
+        <v>0.04312956260474501</v>
       </c>
       <c r="W68" t="n">
-        <v>0.043129562604745</v>
+        <v>0.04312956260474501</v>
       </c>
       <c r="X68" t="n">
         <v>1</v>
       </c>
       <c r="Y68" t="n">
-        <v>75.56512622258113</v>
+        <v>75.56512622258114</v>
       </c>
       <c r="Z68" t="n">
         <v>9</v>
@@ -6061,28 +6061,28 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>214.0942406422302</v>
+        <v>214.0942406422303</v>
       </c>
       <c r="C69" t="n">
         <v>195.8467371567311</v>
       </c>
       <c r="D69" t="n">
-        <v>146.6468161905467</v>
+        <v>146.6468161905466</v>
       </c>
       <c r="E69" t="n">
         <v>245.0466581229155</v>
       </c>
       <c r="F69" t="n">
-        <v>54.87167828512244</v>
+        <v>54.87167828512246</v>
       </c>
       <c r="G69" t="n">
-        <v>59.88974174363473</v>
+        <v>59.88974174363474</v>
       </c>
       <c r="H69" t="n">
         <v>50.25876072668846</v>
       </c>
       <c r="I69" t="n">
-        <v>69.52072276058099</v>
+        <v>69.52072276058101</v>
       </c>
       <c r="J69" t="n">
         <v>126.3546793388604</v>
@@ -6094,43 +6094,43 @@
         <v>147.9843469666629</v>
       </c>
       <c r="M69" t="n">
-        <v>0.05580084957265126</v>
+        <v>0.05580084957265127</v>
       </c>
       <c r="N69" t="n">
         <v>0.008309320739044451</v>
       </c>
       <c r="O69" t="n">
-        <v>0.1138135088801462</v>
+        <v>0.1138135088801463</v>
       </c>
       <c r="P69" t="n">
         <v>0.2091451064804281</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.01359193887047739</v>
+        <v>0.0135919388704774</v>
       </c>
       <c r="R69" t="n">
-        <v>0.626735498597907</v>
+        <v>0.6267354985979071</v>
       </c>
       <c r="S69" t="n">
-        <v>3.264813596684159</v>
+        <v>3.26481359668416</v>
       </c>
       <c r="T69" t="n">
-        <v>0.9848543229687556</v>
+        <v>0.9848543229687561</v>
       </c>
       <c r="U69" t="n">
-        <v>5.544772870399562</v>
+        <v>5.544772870399563</v>
       </c>
       <c r="V69" t="n">
-        <v>0.01422513514670291</v>
+        <v>0.01422513514670292</v>
       </c>
       <c r="W69" t="n">
-        <v>0.01422513514670291</v>
+        <v>0.01422513514670292</v>
       </c>
       <c r="X69" t="n">
         <v>1</v>
       </c>
       <c r="Y69" t="n">
-        <v>76.37159738298652</v>
+        <v>76.37159738298654</v>
       </c>
       <c r="Z69" t="n">
         <v>49</v>
@@ -6161,7 +6161,7 @@
         <v>58.51332937109495</v>
       </c>
       <c r="H70" t="n">
-        <v>54.64477631315522</v>
+        <v>54.64477631315523</v>
       </c>
       <c r="I70" t="n">
         <v>62.38188242903468</v>
@@ -6173,16 +6173,16 @@
         <v>105.7505231542087</v>
       </c>
       <c r="L70" t="n">
-        <v>147.0487040303773</v>
+        <v>147.0487040303774</v>
       </c>
       <c r="M70" t="n">
-        <v>0.05806077627900958</v>
+        <v>0.05806077627900959</v>
       </c>
       <c r="N70" t="n">
-        <v>0.009423926818409815</v>
+        <v>0.009423926818409818</v>
       </c>
       <c r="O70" t="n">
-        <v>0.1168903416248541</v>
+        <v>0.1168903416248542</v>
       </c>
       <c r="P70" t="n">
         <v>0.2039654736897246</v>
@@ -6191,10 +6191,10 @@
         <v>0.0153645923393544</v>
       </c>
       <c r="R70" t="n">
-        <v>0.618245304779183</v>
+        <v>0.6182453047791832</v>
       </c>
       <c r="S70" t="n">
-        <v>3.25104633324576</v>
+        <v>3.251046333245761</v>
       </c>
       <c r="T70" t="n">
         <v>2.604797802511044</v>
@@ -6212,7 +6212,7 @@
         <v>1</v>
       </c>
       <c r="Y70" t="n">
-        <v>76.25664616521362</v>
+        <v>76.25664616521365</v>
       </c>
       <c r="Z70" t="n">
         <v>16</v>
@@ -6228,7 +6228,7 @@
         <v>183.4563403517019</v>
       </c>
       <c r="C71" t="n">
-        <v>148.5812950410716</v>
+        <v>148.5812950410717</v>
       </c>
       <c r="D71" t="n">
         <v>104.5134413412849</v>
@@ -6237,13 +6237,13 @@
         <v>192.6491487408584</v>
       </c>
       <c r="F71" t="n">
-        <v>86.44605339418614</v>
+        <v>86.44605339418615</v>
       </c>
       <c r="G71" t="n">
-        <v>96.03669085460946</v>
+        <v>96.03669085460945</v>
       </c>
       <c r="H71" t="n">
-        <v>81.20293216344363</v>
+        <v>81.20293216344362</v>
       </c>
       <c r="I71" t="n">
         <v>110.8704495457753</v>
@@ -6258,19 +6258,19 @@
         <v>160.1308998105363</v>
       </c>
       <c r="M71" t="n">
-        <v>0.01404215329001335</v>
+        <v>0.01404215329001336</v>
       </c>
       <c r="N71" t="n">
         <v>0.002417355479895621</v>
       </c>
       <c r="O71" t="n">
-        <v>0.02971269109130868</v>
+        <v>0.02971269109130869</v>
       </c>
       <c r="P71" t="n">
-        <v>0.04757644516273927</v>
+        <v>0.04757644516273926</v>
       </c>
       <c r="Q71" t="n">
-        <v>0.009449493632048616</v>
+        <v>0.009449493632048618</v>
       </c>
       <c r="R71" t="n">
         <v>0.1286151130533457</v>
@@ -6294,7 +6294,7 @@
         <v>1</v>
       </c>
       <c r="Y71" t="n">
-        <v>99.16097564697259</v>
+        <v>99.1609756469726</v>
       </c>
       <c r="Z71" t="n">
         <v>4</v>
@@ -6340,7 +6340,7 @@
         <v>149.5092477053341</v>
       </c>
       <c r="M72" t="n">
-        <v>0.09970486469113965</v>
+        <v>0.09970486469113962</v>
       </c>
       <c r="N72" t="n">
         <v>0.01359260316094777</v>
@@ -6352,7 +6352,7 @@
         <v>0.5506740086766594</v>
       </c>
       <c r="Q72" t="n">
-        <v>0.00897272917864291</v>
+        <v>0.008972729178642912</v>
       </c>
       <c r="R72" t="n">
         <v>1.749215385984632</v>
@@ -6477,22 +6477,22 @@
         <v>158.6304321219283</v>
       </c>
       <c r="D74" t="n">
-        <v>72.66874899962264</v>
+        <v>72.66874899962261</v>
       </c>
       <c r="E74" t="n">
-        <v>244.592115244234</v>
+        <v>244.5921152442339</v>
       </c>
       <c r="F74" t="n">
         <v>40.4835192843985</v>
       </c>
       <c r="G74" t="n">
-        <v>42.1870669377215</v>
+        <v>42.18706693772151</v>
       </c>
       <c r="H74" t="n">
         <v>33.99767080028435</v>
       </c>
       <c r="I74" t="n">
-        <v>50.37646307515865</v>
+        <v>50.37646307515867</v>
       </c>
       <c r="J74" t="n">
         <v>107.2749352926961</v>
@@ -6507,7 +6507,7 @@
         <v>0.05330790946922034</v>
       </c>
       <c r="N74" t="n">
-        <v>0.006878560245038559</v>
+        <v>0.00687856024503856</v>
       </c>
       <c r="O74" t="n">
         <v>0.1095634205479257</v>
@@ -6519,16 +6519,16 @@
         <v>0.008694869329370735</v>
       </c>
       <c r="R74" t="n">
-        <v>0.5435910008941626</v>
+        <v>0.5435910008941627</v>
       </c>
       <c r="S74" t="n">
-        <v>-38.64214613843067</v>
+        <v>-38.64214613843066</v>
       </c>
       <c r="T74" t="n">
         <v>-79.91019069364526</v>
       </c>
       <c r="U74" t="n">
-        <v>2.625898416783926</v>
+        <v>2.625898416783933</v>
       </c>
       <c r="V74" t="n">
         <v>0.0275298152247814</v>
@@ -6553,13 +6553,13 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>94.54646848576601</v>
+        <v>94.54646848576603</v>
       </c>
       <c r="C75" t="n">
         <v>86.99670076808778</v>
       </c>
       <c r="D75" t="n">
-        <v>68.615030028283</v>
+        <v>68.61503002828299</v>
       </c>
       <c r="E75" t="n">
         <v>105.3783715078926</v>
@@ -6598,10 +6598,10 @@
         <v>0.03105466129565318</v>
       </c>
       <c r="Q75" t="n">
-        <v>0.008205098550560948</v>
+        <v>0.00820509855056095</v>
       </c>
       <c r="R75" t="n">
-        <v>0.0914443780384967</v>
+        <v>0.09144437803849668</v>
       </c>
       <c r="S75" t="n">
         <v>-17.42662162170728</v>
@@ -6635,7 +6635,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>181.6790999219151</v>
+        <v>181.679099921915</v>
       </c>
       <c r="C76" t="n">
         <v>180.6429532763634</v>
@@ -6647,7 +6647,7 @@
         <v>255.1588663416583</v>
       </c>
       <c r="F76" t="n">
-        <v>32.35810411264713</v>
+        <v>32.35810411264714</v>
       </c>
       <c r="G76" t="n">
         <v>32.64304444017383</v>
@@ -6671,7 +6671,7 @@
         <v>0.06723773050793484</v>
       </c>
       <c r="N76" t="n">
-        <v>0.008839438664743496</v>
+        <v>0.008839438664743494</v>
       </c>
       <c r="O76" t="n">
         <v>0.1375571537125183</v>
@@ -6683,22 +6683,22 @@
         <v>0.00924417335685254</v>
       </c>
       <c r="R76" t="n">
-        <v>0.655107028341667</v>
+        <v>0.6551070283416671</v>
       </c>
       <c r="S76" t="n">
-        <v>-51.92381963044441</v>
+        <v>-51.92381963044442</v>
       </c>
       <c r="T76" t="n">
         <v>-80.34150724405802</v>
       </c>
       <c r="U76" t="n">
-        <v>-23.5061320168308</v>
+        <v>-23.50613201683081</v>
       </c>
       <c r="V76" t="n">
-        <v>0.02424907080875481</v>
+        <v>0.0242490708087548</v>
       </c>
       <c r="W76" t="n">
-        <v>0.02424907080875481</v>
+        <v>0.0242490708087548</v>
       </c>
       <c r="X76" t="n">
         <v>1</v>
@@ -6750,7 +6750,7 @@
         <v>131.026476165366</v>
       </c>
       <c r="M77" t="n">
-        <v>0.01354610825008123</v>
+        <v>0.01354610825008122</v>
       </c>
       <c r="N77" t="n">
         <v>0.005362442093389877</v>
@@ -6759,7 +6759,7 @@
         <v>0.02445436888177059</v>
       </c>
       <c r="P77" t="n">
-        <v>0.0167679748678305</v>
+        <v>0.01676797486783049</v>
       </c>
       <c r="Q77" t="n">
         <v>0.008559739340508486</v>
@@ -6817,7 +6817,7 @@
         <v>63.79161005615261</v>
       </c>
       <c r="H78" t="n">
-        <v>47.74944190721405</v>
+        <v>47.74944190721406</v>
       </c>
       <c r="I78" t="n">
         <v>79.83377820509116</v>
@@ -6835,7 +6835,7 @@
         <v>0.03302794283436643</v>
       </c>
       <c r="N78" t="n">
-        <v>0.0058067246350007</v>
+        <v>0.005806724635000701</v>
       </c>
       <c r="O78" t="n">
         <v>0.06906850177964985</v>
@@ -6920,7 +6920,7 @@
         <v>0.006906163927107253</v>
       </c>
       <c r="O79" t="n">
-        <v>0.06968015549302682</v>
+        <v>0.06968015549302681</v>
       </c>
       <c r="P79" t="n">
         <v>0.119692252325967</v>
@@ -6932,7 +6932,7 @@
         <v>0.3460205961482653</v>
       </c>
       <c r="S79" t="n">
-        <v>2.869579678297741</v>
+        <v>2.86957967829774</v>
       </c>
       <c r="T79" t="n">
         <v>-1.41998992050533</v>
@@ -6963,7 +6963,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>102.4635680135165</v>
+        <v>102.4635680135164</v>
       </c>
       <c r="C80" t="n">
         <v>81.18858534534087</v>
@@ -6975,7 +6975,7 @@
         <v>96.53333460571096</v>
       </c>
       <c r="F80" t="n">
-        <v>50.75241044018447</v>
+        <v>50.75241044018446</v>
       </c>
       <c r="G80" t="n">
         <v>56.60303067393275</v>
@@ -7008,7 +7008,7 @@
         <v>0.0251918940997232</v>
       </c>
       <c r="Q80" t="n">
-        <v>0.008225733703356901</v>
+        <v>0.008225733703356899</v>
       </c>
       <c r="R80" t="n">
         <v>0.07298368284238665</v>
@@ -7032,7 +7032,7 @@
         <v>1</v>
       </c>
       <c r="Y80" t="n">
-        <v>69.98561727905282</v>
+        <v>69.9856172790528</v>
       </c>
       <c r="Z80" t="n">
         <v>4</v>
@@ -7060,13 +7060,13 @@
         <v>69.61412408894613</v>
       </c>
       <c r="G81" t="n">
-        <v>72.57622796334736</v>
+        <v>72.57622796334735</v>
       </c>
       <c r="H81" t="n">
         <v>54.30251033214913</v>
       </c>
       <c r="I81" t="n">
-        <v>90.8499455945456</v>
+        <v>90.84994559454557</v>
       </c>
       <c r="J81" t="n">
         <v>129.4814090689917</v>
@@ -7075,7 +7075,7 @@
         <v>115.8232550863189</v>
       </c>
       <c r="L81" t="n">
-        <v>143.3425488818717</v>
+        <v>143.3425488818716</v>
       </c>
       <c r="M81" t="n">
         <v>0.02442780942329617</v>
@@ -7087,10 +7087,10 @@
         <v>0.04979524739914418</v>
       </c>
       <c r="P81" t="n">
-        <v>0.06084280496946704</v>
+        <v>0.06084280496946703</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.008804875631176878</v>
+        <v>0.008804875631176877</v>
       </c>
       <c r="R81" t="n">
         <v>0.1707218067368158</v>
@@ -7099,10 +7099,10 @@
         <v>1.890878235079883</v>
       </c>
       <c r="T81" t="n">
-        <v>0.6361102366415716</v>
+        <v>0.6361102366415721</v>
       </c>
       <c r="U81" t="n">
-        <v>3.145646233518194</v>
+        <v>3.145646233518193</v>
       </c>
       <c r="V81" t="n">
         <v>0.02522089133940416</v>
@@ -7133,7 +7133,7 @@
         <v>139.9119805119893</v>
       </c>
       <c r="D82" t="n">
-        <v>130.2031699854553</v>
+        <v>130.2031699854552</v>
       </c>
       <c r="E82" t="n">
         <v>149.6207910385233</v>
@@ -7172,19 +7172,19 @@
         <v>0.06085547065928777</v>
       </c>
       <c r="Q82" t="n">
-        <v>0.006142313204050458</v>
+        <v>0.006142313204050459</v>
       </c>
       <c r="R82" t="n">
         <v>0.1726710347675925</v>
       </c>
       <c r="S82" t="n">
-        <v>0.5282475407988007</v>
+        <v>0.5282475407988005</v>
       </c>
       <c r="T82" t="n">
-        <v>-0.2969618115253861</v>
+        <v>-0.2969618115253863</v>
       </c>
       <c r="U82" t="n">
-        <v>1.353456893122988</v>
+        <v>1.353456893122987</v>
       </c>
       <c r="V82" t="n">
         <v>0.01041810408180947</v>
@@ -7196,7 +7196,7 @@
         <v>1</v>
       </c>
       <c r="Y82" t="n">
-        <v>55</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="Z82" t="n">
         <v>4</v>
@@ -7212,22 +7212,22 @@
         <v>100.6987283884684</v>
       </c>
       <c r="C83" t="n">
-        <v>74.9800920147248</v>
+        <v>74.98009201472479</v>
       </c>
       <c r="D83" t="n">
-        <v>58.18956678987427</v>
+        <v>58.18956678987426</v>
       </c>
       <c r="E83" t="n">
-        <v>91.77061723957533</v>
+        <v>91.77061723957532</v>
       </c>
       <c r="F83" t="n">
-        <v>47.85367416439234</v>
+        <v>47.85367416439232</v>
       </c>
       <c r="G83" t="n">
         <v>54.92629916717181</v>
       </c>
       <c r="H83" t="n">
-        <v>50.60751991571921</v>
+        <v>50.6075199157192</v>
       </c>
       <c r="I83" t="n">
         <v>59.24507841862442</v>
@@ -7266,7 +7266,7 @@
         <v>1.872337359231847</v>
       </c>
       <c r="U83" t="n">
-        <v>7.232804979417152</v>
+        <v>7.232804979417153</v>
       </c>
       <c r="V83" t="n">
         <v>0.01983518061281816</v>
@@ -7324,13 +7324,13 @@
         <v>130.0441371052156</v>
       </c>
       <c r="M84" t="n">
-        <v>0.01575162753239507</v>
+        <v>0.01575162753239506</v>
       </c>
       <c r="N84" t="n">
-        <v>0.005012351700370195</v>
+        <v>0.005012351700370194</v>
       </c>
       <c r="O84" t="n">
-        <v>0.02988663925288768</v>
+        <v>0.02988663925288767</v>
       </c>
       <c r="P84" t="n">
         <v>0.02299711547428692</v>
@@ -7373,7 +7373,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>104.4593124158068</v>
+        <v>104.4593124158067</v>
       </c>
       <c r="C85" t="n">
         <v>61.48756181668101</v>
@@ -7388,7 +7388,7 @@
         <v>51.4775166891182</v>
       </c>
       <c r="G85" t="n">
-        <v>63.29474810387778</v>
+        <v>63.29474810387777</v>
       </c>
       <c r="H85" t="n">
         <v>60.11925529683835</v>
@@ -7412,7 +7412,7 @@
         <v>0.004541280335406254</v>
       </c>
       <c r="O85" t="n">
-        <v>0.0386796495735751</v>
+        <v>0.03867964957357509</v>
       </c>
       <c r="P85" t="n">
         <v>0.02432423855685572</v>
@@ -7433,10 +7433,10 @@
         <v>11.23766037441654</v>
       </c>
       <c r="V85" t="n">
-        <v>0.04197613337222166</v>
+        <v>0.04197613337222165</v>
       </c>
       <c r="W85" t="n">
-        <v>0.04197613337222166</v>
+        <v>0.04197613337222165</v>
       </c>
       <c r="X85" t="n">
         <v>1</v>
@@ -7470,19 +7470,19 @@
         <v>59.66868694321361</v>
       </c>
       <c r="G86" t="n">
-        <v>71.80988679624056</v>
+        <v>71.80988679624058</v>
       </c>
       <c r="H86" t="n">
-        <v>65.41654276423439</v>
+        <v>65.41654276423441</v>
       </c>
       <c r="I86" t="n">
-        <v>78.20323082824673</v>
+        <v>78.20323082824675</v>
       </c>
       <c r="J86" t="n">
         <v>128.2874583777616</v>
       </c>
       <c r="K86" t="n">
-        <v>114.417651323826</v>
+        <v>114.4176513238259</v>
       </c>
       <c r="L86" t="n">
         <v>142.4086305932695</v>
@@ -7491,13 +7491,13 @@
         <v>0.0233609656643436</v>
       </c>
       <c r="N86" t="n">
-        <v>0.002449362780309279</v>
+        <v>0.002449362780309278</v>
       </c>
       <c r="O86" t="n">
         <v>0.05212139575059676</v>
       </c>
       <c r="P86" t="n">
-        <v>0.04519340403267276</v>
+        <v>0.04519340403267275</v>
       </c>
       <c r="Q86" t="n">
         <v>0.006924288346200669</v>
@@ -7628,19 +7628,19 @@
         <v>76.54130317218825</v>
       </c>
       <c r="E88" t="n">
-        <v>130.490424443187</v>
+        <v>130.4904244431869</v>
       </c>
       <c r="F88" t="n">
-        <v>62.16216835830645</v>
+        <v>62.16216835830643</v>
       </c>
       <c r="G88" t="n">
-        <v>72.86794563216161</v>
+        <v>72.86794563216159</v>
       </c>
       <c r="H88" t="n">
-        <v>63.02259521517584</v>
+        <v>63.02259521517583</v>
       </c>
       <c r="I88" t="n">
-        <v>82.71329604914737</v>
+        <v>82.71329604914736</v>
       </c>
       <c r="J88" t="n">
         <v>128.2096598699533</v>
@@ -7652,7 +7652,7 @@
         <v>140.9751745851604</v>
       </c>
       <c r="M88" t="n">
-        <v>0.02030090046102806</v>
+        <v>0.02030090046102807</v>
       </c>
       <c r="N88" t="n">
         <v>0.005354567853456634</v>
@@ -7707,7 +7707,7 @@
         <v>182.9314813663034</v>
       </c>
       <c r="D89" t="n">
-        <v>97.79854259990952</v>
+        <v>97.7985425999095</v>
       </c>
       <c r="E89" t="n">
         <v>268.0644201326973</v>
@@ -7740,7 +7740,7 @@
         <v>0.008222181655259772</v>
       </c>
       <c r="O89" t="n">
-        <v>0.0977126599345343</v>
+        <v>0.09771265993453433</v>
       </c>
       <c r="P89" t="n">
         <v>0.196508065231537</v>
@@ -7770,7 +7770,7 @@
         <v>1</v>
       </c>
       <c r="Y89" t="n">
-        <v>77.6813602242361</v>
+        <v>77.68136022423612</v>
       </c>
       <c r="Z89" t="n">
         <v>25</v>
@@ -7795,7 +7795,7 @@
         <v>132.9919336081852</v>
       </c>
       <c r="F90" t="n">
-        <v>44.62740964596922</v>
+        <v>44.62740964596921</v>
       </c>
       <c r="G90" t="n">
         <v>48.96610173717133</v>
@@ -7810,13 +7810,13 @@
         <v>107.4663435326201</v>
       </c>
       <c r="K90" t="n">
-        <v>92.60130807536547</v>
+        <v>92.60130807536545</v>
       </c>
       <c r="L90" t="n">
         <v>123.4289645085261</v>
       </c>
       <c r="M90" t="n">
-        <v>0.03267082651950768</v>
+        <v>0.03267082651950767</v>
       </c>
       <c r="N90" t="n">
         <v>0.005631868766419892</v>
@@ -7877,19 +7877,19 @@
         <v>228.271830467012</v>
       </c>
       <c r="F91" t="n">
-        <v>98.23035690868274</v>
+        <v>98.23035690868272</v>
       </c>
       <c r="G91" t="n">
-        <v>103.1068370417309</v>
+        <v>103.106837041731</v>
       </c>
       <c r="H91" t="n">
-        <v>95.04210897905023</v>
+        <v>95.04210897905025</v>
       </c>
       <c r="I91" t="n">
         <v>111.1715651044117</v>
       </c>
       <c r="J91" t="n">
-        <v>158.715511648101</v>
+        <v>158.7155116481011</v>
       </c>
       <c r="K91" t="n">
         <v>144.7877562534795</v>
@@ -7913,7 +7913,7 @@
         <v>0.01550755140524029</v>
       </c>
       <c r="R91" t="n">
-        <v>0.2775488439742105</v>
+        <v>0.2775488439742106</v>
       </c>
       <c r="S91" t="n">
         <v>4.095763219346411</v>
@@ -7934,7 +7934,7 @@
         <v>1</v>
       </c>
       <c r="Y91" t="n">
-        <v>89.11818626109884</v>
+        <v>89.11818626109883</v>
       </c>
       <c r="Z91" t="n">
         <v>10</v>
@@ -7953,22 +7953,22 @@
         <v>212.5825446844803</v>
       </c>
       <c r="D92" t="n">
-        <v>178.9108202730103</v>
+        <v>178.9108202730102</v>
       </c>
       <c r="E92" t="n">
         <v>246.2542690959503</v>
       </c>
       <c r="F92" t="n">
-        <v>64.94187459052031</v>
+        <v>64.94187459052033</v>
       </c>
       <c r="G92" t="n">
-        <v>64.94187459052031</v>
+        <v>64.94187459052033</v>
       </c>
       <c r="H92" t="n">
-        <v>57.81202523850588</v>
+        <v>57.8120252385059</v>
       </c>
       <c r="I92" t="n">
-        <v>72.07172394253475</v>
+        <v>72.07172394253476</v>
       </c>
       <c r="J92" t="n">
         <v>128.1873105859924</v>
@@ -7980,10 +7980,10 @@
         <v>147.2356695889354</v>
       </c>
       <c r="M92" t="n">
-        <v>0.04317782963393701</v>
+        <v>0.04317782963393702</v>
       </c>
       <c r="N92" t="n">
-        <v>0.007437329298174474</v>
+        <v>0.007437329298174476</v>
       </c>
       <c r="O92" t="n">
         <v>0.08746532627288735</v>
@@ -8007,16 +8007,16 @@
         <v>0</v>
       </c>
       <c r="V92" t="n">
-        <v>0.04073803874033432</v>
+        <v>0.04073803874033433</v>
       </c>
       <c r="W92" t="n">
-        <v>0.04073803874033432</v>
+        <v>0.04073803874033433</v>
       </c>
       <c r="X92" t="n">
         <v>1</v>
       </c>
       <c r="Y92" t="n">
-        <v>81.4207979064941</v>
+        <v>81.42079790649412</v>
       </c>
       <c r="Z92" t="n">
         <v>3</v>
@@ -8147,7 +8147,7 @@
         <v>0.02043766950380553</v>
       </c>
       <c r="N94" t="n">
-        <v>0.004779308069865847</v>
+        <v>0.004779308069865848</v>
       </c>
       <c r="O94" t="n">
         <v>0.04155973013505951</v>
@@ -8165,10 +8165,10 @@
         <v>3.799782663014903</v>
       </c>
       <c r="T94" t="n">
-        <v>1.154953224975639</v>
+        <v>1.154953224975641</v>
       </c>
       <c r="U94" t="n">
-        <v>6.444612101054167</v>
+        <v>6.444612101054166</v>
       </c>
       <c r="V94" t="n">
         <v>0.02313305167578536</v>
@@ -8193,28 +8193,28 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>96.90864993950433</v>
+        <v>96.90864993950434</v>
       </c>
       <c r="C95" t="n">
-        <v>74.21629323550401</v>
+        <v>74.21629323550403</v>
       </c>
       <c r="D95" t="n">
-        <v>59.35394142943404</v>
+        <v>59.35394142943406</v>
       </c>
       <c r="E95" t="n">
-        <v>89.07864504157398</v>
+        <v>89.07864504157399</v>
       </c>
       <c r="F95" t="n">
-        <v>53.69509821947065</v>
+        <v>53.69509821947066</v>
       </c>
       <c r="G95" t="n">
-        <v>59.93549631307073</v>
+        <v>59.93549631307074</v>
       </c>
       <c r="H95" t="n">
-        <v>51.94490091159364</v>
+        <v>51.94490091159366</v>
       </c>
       <c r="I95" t="n">
-        <v>67.92609171454782</v>
+        <v>67.92609171454784</v>
       </c>
       <c r="J95" t="n">
         <v>113.5576107242979</v>
@@ -8223,19 +8223,19 @@
         <v>102.5974340457654</v>
       </c>
       <c r="L95" t="n">
-        <v>124.4292557778982</v>
+        <v>124.4292557778983</v>
       </c>
       <c r="M95" t="n">
-        <v>0.01586047235740842</v>
+        <v>0.01586047235740843</v>
       </c>
       <c r="N95" t="n">
-        <v>0.006093121083572016</v>
+        <v>0.006093121083572018</v>
       </c>
       <c r="O95" t="n">
-        <v>0.02896668264244358</v>
+        <v>0.02896668264244359</v>
       </c>
       <c r="P95" t="n">
-        <v>0.01877372904557254</v>
+        <v>0.01877372904557255</v>
       </c>
       <c r="Q95" t="n">
         <v>0.008567405467626361</v>
@@ -8244,13 +8244,13 @@
         <v>0.05611518252043873</v>
       </c>
       <c r="S95" t="n">
-        <v>4.486377249952093</v>
+        <v>4.486377249952094</v>
       </c>
       <c r="T95" t="n">
-        <v>0.7326678157717583</v>
+        <v>0.7326678157717588</v>
       </c>
       <c r="U95" t="n">
-        <v>8.240086684132427</v>
+        <v>8.240086684132429</v>
       </c>
       <c r="V95" t="n">
         <v>0.02263227446061343</v>
@@ -8278,16 +8278,16 @@
         <v>138.3756736756322</v>
       </c>
       <c r="C96" t="n">
-        <v>92.29082234367419</v>
+        <v>92.29082234367415</v>
       </c>
       <c r="D96" t="n">
-        <v>35.63013925584701</v>
+        <v>35.63013925584699</v>
       </c>
       <c r="E96" t="n">
-        <v>148.9515054315014</v>
+        <v>148.9515054315013</v>
       </c>
       <c r="F96" t="n">
-        <v>75.09596320132886</v>
+        <v>75.09596320132884</v>
       </c>
       <c r="G96" t="n">
         <v>87.7692973176173</v>
@@ -8305,7 +8305,7 @@
         <v>128.7664580909565</v>
       </c>
       <c r="L96" t="n">
-        <v>147.5918266662968</v>
+        <v>147.5918266662967</v>
       </c>
       <c r="M96" t="n">
         <v>0.01161449532909637</v>
@@ -8375,10 +8375,10 @@
         <v>64.22592181759683</v>
       </c>
       <c r="H97" t="n">
-        <v>55.75276845533185</v>
+        <v>55.75276845533186</v>
       </c>
       <c r="I97" t="n">
-        <v>72.69907517986181</v>
+        <v>72.69907517986179</v>
       </c>
       <c r="J97" t="n">
         <v>121.9227893814793</v>
@@ -8402,7 +8402,7 @@
         <v>0.05100145419049692</v>
       </c>
       <c r="Q97" t="n">
-        <v>0.007178058215559461</v>
+        <v>0.00717805821555946</v>
       </c>
       <c r="R97" t="n">
         <v>0.1435135916716826</v>
@@ -8463,13 +8463,13 @@
         <v>80.07066501470894</v>
       </c>
       <c r="J98" t="n">
-        <v>122.1818760862949</v>
+        <v>122.181876086295</v>
       </c>
       <c r="K98" t="n">
         <v>110.4420944689975</v>
       </c>
       <c r="L98" t="n">
-        <v>134.636591245297</v>
+        <v>134.6365912452971</v>
       </c>
       <c r="M98" t="n">
         <v>0.01974463670617732</v>
@@ -8490,13 +8490,13 @@
         <v>0.1020309740561361</v>
       </c>
       <c r="S98" t="n">
-        <v>5.10822780918186</v>
+        <v>5.108227809181858</v>
       </c>
       <c r="T98" t="n">
-        <v>1.536710899490295</v>
+        <v>1.536710899490294</v>
       </c>
       <c r="U98" t="n">
-        <v>8.679744718873424</v>
+        <v>8.679744718873422</v>
       </c>
       <c r="V98" t="n">
         <v>0.01427733640412051</v>
@@ -8527,7 +8527,7 @@
         <v>113.1775248211505</v>
       </c>
       <c r="D99" t="n">
-        <v>90.44100101949184</v>
+        <v>90.44100101949182</v>
       </c>
       <c r="E99" t="n">
         <v>135.9140486228091</v>
@@ -8545,13 +8545,13 @@
         <v>88.73236066473103</v>
       </c>
       <c r="J99" t="n">
-        <v>134.0045602182841</v>
+        <v>134.004560218284</v>
       </c>
       <c r="K99" t="n">
         <v>121.8373894476993</v>
       </c>
       <c r="L99" t="n">
-        <v>146.9042018880654</v>
+        <v>146.9042018880655</v>
       </c>
       <c r="M99" t="n">
         <v>0.01953102792490467</v>
@@ -8575,10 +8575,10 @@
         <v>9.756618981545055</v>
       </c>
       <c r="T99" t="n">
-        <v>7.472346214856965</v>
+        <v>7.472346214856964</v>
       </c>
       <c r="U99" t="n">
-        <v>12.04089174823314</v>
+        <v>12.04089174823315</v>
       </c>
       <c r="V99" t="n">
         <v>0.01450413063066497</v>
@@ -8633,7 +8633,7 @@
         <v>111.9890318062021</v>
       </c>
       <c r="L100" t="n">
-        <v>133.9414479024336</v>
+        <v>133.9414479024335</v>
       </c>
       <c r="M100" t="n">
         <v>0.01621195557112087</v>
@@ -8685,7 +8685,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>97.59936954494468</v>
+        <v>97.59936954494466</v>
       </c>
       <c r="C101" t="n">
         <v>72.54889166813942</v>
@@ -8697,7 +8697,7 @@
         <v>84.82246006382307</v>
       </c>
       <c r="F101" t="n">
-        <v>50.49091480872923</v>
+        <v>50.49091480872922</v>
       </c>
       <c r="G101" t="n">
         <v>57.37979622485068</v>
@@ -8709,40 +8709,40 @@
         <v>61.21873061084621</v>
       </c>
       <c r="J101" t="n">
-        <v>112.0046573636948</v>
+        <v>112.0046573636947</v>
       </c>
       <c r="K101" t="n">
-        <v>99.98595412648288</v>
+        <v>99.98595412648287</v>
       </c>
       <c r="L101" t="n">
-        <v>123.6763547758255</v>
+        <v>123.6763547758254</v>
       </c>
       <c r="M101" t="n">
         <v>0.01915042527418456</v>
       </c>
       <c r="N101" t="n">
-        <v>0.005903378219024221</v>
+        <v>0.00590337821902422</v>
       </c>
       <c r="O101" t="n">
         <v>0.03696064290882949</v>
       </c>
       <c r="P101" t="n">
-        <v>0.02282063787808342</v>
+        <v>0.02282063787808341</v>
       </c>
       <c r="Q101" t="n">
-        <v>0.00827189002104793</v>
+        <v>0.008271890021047928</v>
       </c>
       <c r="R101" t="n">
-        <v>0.06701219896736633</v>
+        <v>0.06701219896736632</v>
       </c>
       <c r="S101" t="n">
-        <v>4.286664460931752</v>
+        <v>4.286664460931751</v>
       </c>
       <c r="T101" t="n">
-        <v>2.360867717180266</v>
+        <v>2.360867717180265</v>
       </c>
       <c r="U101" t="n">
-        <v>6.212461204683239</v>
+        <v>6.212461204683238</v>
       </c>
       <c r="V101" t="n">
         <v>0.02137260780735586</v>
@@ -8754,7 +8754,7 @@
         <v>1</v>
       </c>
       <c r="Y101" t="n">
-        <v>86.1588478506451</v>
+        <v>86.15884785064509</v>
       </c>
       <c r="Z101" t="n">
         <v>14</v>
@@ -8770,7 +8770,7 @@
         <v>121.6910619431209</v>
       </c>
       <c r="C102" t="n">
-        <v>82.675984806155</v>
+        <v>82.67598480615499</v>
       </c>
       <c r="D102" t="n">
         <v>62.38626340773006</v>
@@ -8779,13 +8779,13 @@
         <v>102.9657062045799</v>
       </c>
       <c r="F102" t="n">
-        <v>56.34397449659641</v>
+        <v>56.3439744965964</v>
       </c>
       <c r="G102" t="n">
-        <v>67.07312070926204</v>
+        <v>67.07312070926203</v>
       </c>
       <c r="H102" t="n">
-        <v>63.00528025864644</v>
+        <v>63.00528025864642</v>
       </c>
       <c r="I102" t="n">
         <v>71.14096115987763</v>
@@ -8803,13 +8803,13 @@
         <v>0.01854394347285594</v>
       </c>
       <c r="N102" t="n">
-        <v>0.00470846823008368</v>
+        <v>0.004708468230083679</v>
       </c>
       <c r="O102" t="n">
         <v>0.03724432013144011</v>
       </c>
       <c r="P102" t="n">
-        <v>0.02971534080691601</v>
+        <v>0.029715340806916</v>
       </c>
       <c r="Q102" t="n">
         <v>0.007354451256208263</v>
@@ -8818,19 +8818,19 @@
         <v>0.08264902759725631</v>
       </c>
       <c r="S102" t="n">
-        <v>8.498836344779082</v>
+        <v>8.498836344779084</v>
       </c>
       <c r="T102" t="n">
-        <v>5.49760124196538</v>
+        <v>5.497601241965381</v>
       </c>
       <c r="U102" t="n">
-        <v>11.50007144759278</v>
+        <v>11.50007144759279</v>
       </c>
       <c r="V102" t="n">
-        <v>0.02702648294392155</v>
+        <v>0.02702648294392156</v>
       </c>
       <c r="W102" t="n">
-        <v>0.02702648294392155</v>
+        <v>0.02702648294392156</v>
       </c>
       <c r="X102" t="n">
         <v>1</v>
@@ -8855,10 +8855,10 @@
         <v>81.55088053567889</v>
       </c>
       <c r="D103" t="n">
-        <v>64.27553421111159</v>
+        <v>64.27553421111161</v>
       </c>
       <c r="E103" t="n">
-        <v>98.82622686024618</v>
+        <v>98.82622686024617</v>
       </c>
       <c r="F103" t="n">
         <v>50.18403076768174</v>
@@ -8882,16 +8882,16 @@
         <v>123.8499659241255</v>
       </c>
       <c r="M103" t="n">
-        <v>0.02046618416521045</v>
+        <v>0.02046618416521046</v>
       </c>
       <c r="N103" t="n">
-        <v>0.00571509337563021</v>
+        <v>0.005715093375630211</v>
       </c>
       <c r="O103" t="n">
         <v>0.03988269277232358</v>
       </c>
       <c r="P103" t="n">
-        <v>0.02595322707092048</v>
+        <v>0.02595322707092049</v>
       </c>
       <c r="Q103" t="n">
         <v>0.008196373251903987</v>
@@ -8949,13 +8949,13 @@
         <v>109.0358552167522</v>
       </c>
       <c r="H104" t="n">
-        <v>99.4832028873499</v>
+        <v>99.48320288734988</v>
       </c>
       <c r="I104" t="n">
         <v>118.5885075461545</v>
       </c>
       <c r="J104" t="n">
-        <v>161.3158127537124</v>
+        <v>161.3158127537125</v>
       </c>
       <c r="K104" t="n">
         <v>148.8532022480333</v>
@@ -8985,7 +8985,7 @@
         <v>10.97739928856033</v>
       </c>
       <c r="T104" t="n">
-        <v>7.758467414086324</v>
+        <v>7.758467414086326</v>
       </c>
       <c r="U104" t="n">
         <v>14.19633116303434</v>
@@ -9000,7 +9000,7 @@
         <v>1</v>
       </c>
       <c r="Y104" t="n">
-        <v>76.61885600176126</v>
+        <v>76.61885600176124</v>
       </c>
       <c r="Z104" t="n">
         <v>13</v>
@@ -9043,7 +9043,7 @@
         <v>110.683563866863</v>
       </c>
       <c r="L105" t="n">
-        <v>132.6835638668629</v>
+        <v>132.683563866863</v>
       </c>
       <c r="M105" t="n">
         <v>0.01616969147103211</v>
@@ -9140,7 +9140,7 @@
         <v>0.0797238592253624</v>
       </c>
       <c r="Q106" t="n">
-        <v>0.01852974796959175</v>
+        <v>0.01852974796959174</v>
       </c>
       <c r="R106" t="n">
         <v>0.2188311291677606</v>
@@ -9195,19 +9195,19 @@
         <v>85.77958607162752</v>
       </c>
       <c r="H107" t="n">
-        <v>63.69728958379154</v>
+        <v>63.69728958379156</v>
       </c>
       <c r="I107" t="n">
         <v>107.8618825594635</v>
       </c>
       <c r="J107" t="n">
-        <v>137.6104025939814</v>
+        <v>137.6104025939813</v>
       </c>
       <c r="K107" t="n">
         <v>128.0176590065919</v>
       </c>
       <c r="L107" t="n">
-        <v>146.7295442788104</v>
+        <v>146.7295442788105</v>
       </c>
       <c r="M107" t="n">
         <v>0.0115344090005139</v>
@@ -9219,7 +9219,7 @@
         <v>0.01976539763151987</v>
       </c>
       <c r="P107" t="n">
-        <v>0.03137041632603192</v>
+        <v>0.03137041632603191</v>
       </c>
       <c r="Q107" t="n">
         <v>0.01081543959538245</v>
@@ -9265,19 +9265,19 @@
         <v>138.7353667491495</v>
       </c>
       <c r="D108" t="n">
-        <v>91.06639275952269</v>
+        <v>91.06639275952267</v>
       </c>
       <c r="E108" t="n">
         <v>186.4043407387763</v>
       </c>
       <c r="F108" t="n">
-        <v>78.42631224111746</v>
+        <v>78.42631224111747</v>
       </c>
       <c r="G108" t="n">
-        <v>87.94282533113881</v>
+        <v>87.94282533113879</v>
       </c>
       <c r="H108" t="n">
-        <v>69.04756839615604</v>
+        <v>69.04756839615602</v>
       </c>
       <c r="I108" t="n">
         <v>106.8380822661216</v>
@@ -9286,7 +9286,7 @@
         <v>141.545473598503</v>
       </c>
       <c r="K108" t="n">
-        <v>129.9029058692952</v>
+        <v>129.9029058692953</v>
       </c>
       <c r="L108" t="n">
         <v>153.7466357903127</v>
@@ -9295,25 +9295,25 @@
         <v>0.017494520187821</v>
       </c>
       <c r="N108" t="n">
-        <v>0.004569243792870696</v>
+        <v>0.004569243792870697</v>
       </c>
       <c r="O108" t="n">
-        <v>0.0352731701570235</v>
+        <v>0.03527317015702349</v>
       </c>
       <c r="P108" t="n">
-        <v>0.05109145422460157</v>
+        <v>0.05109145422460159</v>
       </c>
       <c r="Q108" t="n">
-        <v>0.009365324072054038</v>
+        <v>0.009365324072054039</v>
       </c>
       <c r="R108" t="n">
         <v>0.141168690067351</v>
       </c>
       <c r="S108" t="n">
-        <v>8.35003956919752</v>
+        <v>8.350039569197522</v>
       </c>
       <c r="T108" t="n">
-        <v>6.166438117881371</v>
+        <v>6.166438117881372</v>
       </c>
       <c r="U108" t="n">
         <v>10.53364102051367</v>
@@ -9328,7 +9328,7 @@
         <v>1</v>
       </c>
       <c r="Y108" t="n">
-        <v>75.2116952055585</v>
+        <v>75.21169520555851</v>
       </c>
       <c r="Z108" t="n">
         <v>5</v>
@@ -9347,13 +9347,13 @@
         <v>177.5661179108791</v>
       </c>
       <c r="D109" t="n">
-        <v>147.3666496690459</v>
+        <v>147.366649669046</v>
       </c>
       <c r="E109" t="n">
         <v>207.7655861527123</v>
       </c>
       <c r="F109" t="n">
-        <v>94.45566923756962</v>
+        <v>94.45566923756964</v>
       </c>
       <c r="G109" t="n">
         <v>104.8499551226648</v>
@@ -9368,13 +9368,13 @@
         <v>158.2668404935949</v>
       </c>
       <c r="K109" t="n">
-        <v>145.2025656685871</v>
+        <v>145.202565668587</v>
       </c>
       <c r="L109" t="n">
-        <v>171.330294108176</v>
+        <v>171.3302941081761</v>
       </c>
       <c r="M109" t="n">
-        <v>0.01798585537221124</v>
+        <v>0.01798585537221125</v>
       </c>
       <c r="N109" t="n">
         <v>0.003929747256223651</v>
@@ -9383,19 +9383,19 @@
         <v>0.0371771273165724</v>
       </c>
       <c r="P109" t="n">
-        <v>0.07936426736451015</v>
+        <v>0.07936426736451016</v>
       </c>
       <c r="Q109" t="n">
-        <v>0.012750089670886</v>
+        <v>0.01275008967088601</v>
       </c>
       <c r="R109" t="n">
-        <v>0.2186342838885584</v>
+        <v>0.2186342838885585</v>
       </c>
       <c r="S109" t="n">
         <v>11.84247208427066</v>
       </c>
       <c r="T109" t="n">
-        <v>9.889709983404305</v>
+        <v>9.889709983404309</v>
       </c>
       <c r="U109" t="n">
         <v>13.79523418513701</v>
@@ -9426,31 +9426,31 @@
         <v>93.59514967376928</v>
       </c>
       <c r="C110" t="n">
-        <v>74.16047842456383</v>
+        <v>74.16047842456385</v>
       </c>
       <c r="D110" t="n">
-        <v>65.23154053226064</v>
+        <v>65.23154053226065</v>
       </c>
       <c r="E110" t="n">
-        <v>83.08941631686703</v>
+        <v>83.08941631686704</v>
       </c>
       <c r="F110" t="n">
         <v>49.21077782227692</v>
       </c>
       <c r="G110" t="n">
-        <v>54.55531241580842</v>
+        <v>54.55531241580843</v>
       </c>
       <c r="H110" t="n">
         <v>49.70638119984088</v>
       </c>
       <c r="I110" t="n">
-        <v>59.40424363177597</v>
+        <v>59.40424363177598</v>
       </c>
       <c r="J110" t="n">
         <v>109.2066558283996</v>
       </c>
       <c r="K110" t="n">
-        <v>97.12769540701703</v>
+        <v>97.12769540701704</v>
       </c>
       <c r="L110" t="n">
         <v>120.8988599683248</v>
@@ -9459,7 +9459,7 @@
         <v>0.01969596027802956</v>
       </c>
       <c r="N110" t="n">
-        <v>0.006021837430391914</v>
+        <v>0.006021837430391915</v>
       </c>
       <c r="O110" t="n">
         <v>0.03796810541556483</v>
@@ -9468,10 +9468,10 @@
         <v>0.022059149431249</v>
       </c>
       <c r="Q110" t="n">
-        <v>0.008437912041278726</v>
+        <v>0.008437912041278728</v>
       </c>
       <c r="R110" t="n">
-        <v>0.06532722957850157</v>
+        <v>0.06532722957850158</v>
       </c>
       <c r="S110" t="n">
         <v>3.181229387066385</v>
@@ -9480,7 +9480,7 @@
         <v>1.263804263152924</v>
       </c>
       <c r="U110" t="n">
-        <v>5.098654510979846</v>
+        <v>5.098654510979847</v>
       </c>
       <c r="V110" t="n">
         <v>0.01703626756441336</v>
@@ -9505,10 +9505,10 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>212.5010558433806</v>
+        <v>212.5010558433805</v>
       </c>
       <c r="C111" t="n">
-        <v>193.9755234436288</v>
+        <v>193.9755234436287</v>
       </c>
       <c r="D111" t="n">
         <v>160.6121279771821</v>
@@ -9520,49 +9520,49 @@
         <v>105.0736550333621</v>
       </c>
       <c r="G111" t="n">
-        <v>110.1681764432939</v>
+        <v>110.1681764432938</v>
       </c>
       <c r="H111" t="n">
-        <v>99.47286010634872</v>
+        <v>99.47286010634868</v>
       </c>
       <c r="I111" t="n">
         <v>120.863492780239</v>
       </c>
       <c r="J111" t="n">
-        <v>158.9481219221629</v>
+        <v>158.9481219221628</v>
       </c>
       <c r="K111" t="n">
         <v>147.0925864881156</v>
       </c>
       <c r="L111" t="n">
-        <v>169.8001676214509</v>
+        <v>169.8001676214508</v>
       </c>
       <c r="M111" t="n">
         <v>0.01154790742408325</v>
       </c>
       <c r="N111" t="n">
-        <v>0.002447102178136515</v>
+        <v>0.002447102178136514</v>
       </c>
       <c r="O111" t="n">
-        <v>0.0239334108693986</v>
+        <v>0.02393341086939859</v>
       </c>
       <c r="P111" t="n">
-        <v>0.05327485149327312</v>
+        <v>0.05327485149327311</v>
       </c>
       <c r="Q111" t="n">
         <v>0.01289451149888434</v>
       </c>
       <c r="R111" t="n">
-        <v>0.1454206355350196</v>
+        <v>0.1454206355350195</v>
       </c>
       <c r="S111" t="n">
-        <v>4.315202032293513</v>
+        <v>4.315202032293512</v>
       </c>
       <c r="T111" t="n">
         <v>2.305354034011527</v>
       </c>
       <c r="U111" t="n">
-        <v>6.325050030575499</v>
+        <v>6.325050030575497</v>
       </c>
       <c r="V111" t="n">
         <v>0.02320276161171361</v>
@@ -9611,7 +9611,7 @@
         <v>42.76376661091405</v>
       </c>
       <c r="J112" t="n">
-        <v>100.8225147601762</v>
+        <v>100.8225147601761</v>
       </c>
       <c r="K112" t="n">
         <v>83.0867876463585</v>

</xml_diff>